<commit_message>
Split spirometry row into fev1, fvc, fev1_fvc concept rows
Add SPIROMETRY_OMOP_MAP and parse_observation_set_yaml() to 01_parse_yaml_phvs.py
to walk MeasurementObservationSet YAML structure and emit one row per spirometry
concept based on observation_type OMOP codes. Other spirometry measurements
(% predicted) are ignored. Table now has 105 rows (was 103 after synonym merges).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tables/before_table.xlsx
+++ b/tables/before_table.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U104"/>
+  <dimension ref="A1:U106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3585,160 +3585,160 @@
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>fibrin</t>
+          <t>fev1</t>
         </is>
       </c>
       <c r="B46" s="7" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="C46" s="7" t="n">
-        <v>15767</v>
+        <v>87503</v>
       </c>
       <c r="D46" s="7" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E46" s="7" t="n">
-        <v>10916</v>
+        <v>64098</v>
       </c>
       <c r="F46" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G46" s="7" t="n">
-        <v>25124</v>
+        <v>31282</v>
       </c>
       <c r="H46" s="7" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I46" s="7" t="n">
-        <v>0</v>
+        <v>82063</v>
       </c>
       <c r="J46" s="7" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="K46" s="7" t="n">
-        <v>53858</v>
+        <v>124086</v>
       </c>
       <c r="L46" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M46" s="7" t="n">
-        <v>0</v>
+        <v>34509</v>
       </c>
       <c r="N46" s="7" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="O46" s="7" t="n">
-        <v>0</v>
+        <v>14702</v>
       </c>
       <c r="P46" s="7" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="Q46" s="7" t="n">
-        <v>21121</v>
+        <v>12201</v>
       </c>
       <c r="R46" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S46" s="7" t="n">
-        <v>46006</v>
+        <v>0</v>
       </c>
       <c r="T46" s="5" t="n">
-        <v>39</v>
+        <v>94</v>
       </c>
       <c r="U46" s="5" t="n">
-        <v>172792</v>
+        <v>450444</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>fruit_serving</t>
+          <t>fev1_fvc</t>
         </is>
       </c>
       <c r="B47" s="7" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="C47" s="7" t="n">
-        <v>175886</v>
+        <v>82611</v>
       </c>
       <c r="D47" s="7" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="E47" s="7" t="n">
-        <v>40644</v>
+        <v>0</v>
       </c>
       <c r="F47" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G47" s="7" t="n">
-        <v>5690</v>
+        <v>9673</v>
       </c>
       <c r="H47" s="7" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I47" s="7" t="n">
-        <v>0</v>
+        <v>82063</v>
       </c>
       <c r="J47" s="7" t="n">
-        <v>130</v>
+        <v>24</v>
       </c>
       <c r="K47" s="7" t="n">
-        <v>375548</v>
+        <v>111182</v>
       </c>
       <c r="L47" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M47" s="7" t="n">
-        <v>0</v>
+        <v>34422</v>
       </c>
       <c r="N47" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O47" s="7" t="n">
-        <v>0</v>
+        <v>11044</v>
       </c>
       <c r="P47" s="7" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="Q47" s="7" t="n">
-        <v>8534</v>
+        <v>12550</v>
       </c>
       <c r="R47" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S47" s="7" t="n">
-        <v>1018181</v>
+        <v>0</v>
       </c>
       <c r="T47" s="5" t="n">
-        <v>168</v>
+        <v>54</v>
       </c>
       <c r="U47" s="5" t="n">
-        <v>1624483</v>
+        <v>343545</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>glucose_bld</t>
+          <t>fibrin</t>
         </is>
       </c>
       <c r="B48" s="7" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="C48" s="7" t="n">
-        <v>211779</v>
+        <v>15767</v>
       </c>
       <c r="D48" s="7" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E48" s="7" t="n">
-        <v>6763</v>
+        <v>10916</v>
       </c>
       <c r="F48" s="7" t="n">
         <v>7</v>
       </c>
       <c r="G48" s="7" t="n">
-        <v>25155</v>
+        <v>25124</v>
       </c>
       <c r="H48" s="7" t="n">
         <v>0</v>
@@ -3747,10 +3747,10 @@
         <v>0</v>
       </c>
       <c r="J48" s="7" t="n">
-        <v>102</v>
+        <v>15</v>
       </c>
       <c r="K48" s="7" t="n">
-        <v>292594</v>
+        <v>53858</v>
       </c>
       <c r="L48" s="7" t="n">
         <v>0</v>
@@ -3759,53 +3759,53 @@
         <v>0</v>
       </c>
       <c r="N48" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="O48" s="7" t="n">
-        <v>10187</v>
+        <v>0</v>
       </c>
       <c r="P48" s="7" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="Q48" s="7" t="n">
-        <v>358</v>
+        <v>21121</v>
       </c>
       <c r="R48" s="7" t="n">
         <v>3</v>
       </c>
       <c r="S48" s="7" t="n">
-        <v>46598</v>
+        <v>46006</v>
       </c>
       <c r="T48" s="5" t="n">
-        <v>139</v>
+        <v>39</v>
       </c>
       <c r="U48" s="5" t="n">
-        <v>593434</v>
+        <v>172792</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>hdl</t>
+          <t>fruit_serving</t>
         </is>
       </c>
       <c r="B49" s="7" t="n">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="C49" s="7" t="n">
-        <v>282573</v>
+        <v>175886</v>
       </c>
       <c r="D49" s="7" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E49" s="7" t="n">
-        <v>16570</v>
+        <v>40644</v>
       </c>
       <c r="F49" s="7" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G49" s="7" t="n">
-        <v>29869</v>
+        <v>5690</v>
       </c>
       <c r="H49" s="7" t="n">
         <v>0</v>
@@ -3814,199 +3814,199 @@
         <v>0</v>
       </c>
       <c r="J49" s="7" t="n">
-        <v>52</v>
+        <v>130</v>
       </c>
       <c r="K49" s="7" t="n">
-        <v>148153</v>
+        <v>375548</v>
       </c>
       <c r="L49" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M49" s="7" t="n">
-        <v>23652</v>
+        <v>0</v>
       </c>
       <c r="N49" s="7" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="O49" s="7" t="n">
-        <v>32797</v>
+        <v>0</v>
       </c>
       <c r="P49" s="7" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="Q49" s="7" t="n">
-        <v>74205</v>
+        <v>8534</v>
       </c>
       <c r="R49" s="7" t="n">
         <v>3</v>
       </c>
       <c r="S49" s="7" t="n">
-        <v>46573</v>
+        <v>1018181</v>
       </c>
       <c r="T49" s="5" t="n">
-        <v>131</v>
+        <v>168</v>
       </c>
       <c r="U49" s="5" t="n">
-        <v>654392</v>
+        <v>1624483</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>hemat</t>
+          <t>fvc</t>
         </is>
       </c>
       <c r="B50" s="7" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C50" s="7" t="n">
-        <v>61658</v>
+        <v>73309</v>
       </c>
       <c r="D50" s="7" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="E50" s="7" t="n">
-        <v>3582</v>
+        <v>57425</v>
       </c>
       <c r="F50" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G50" s="7" t="n">
-        <v>25115</v>
+        <v>24859</v>
       </c>
       <c r="H50" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I50" s="7" t="n">
-        <v>53674</v>
+        <v>82067</v>
       </c>
       <c r="J50" s="7" t="n">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="K50" s="7" t="n">
-        <v>154499</v>
+        <v>127166</v>
       </c>
       <c r="L50" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M50" s="7" t="n">
-        <v>23567</v>
+        <v>34509</v>
       </c>
       <c r="N50" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O50" s="7" t="n">
-        <v>3746</v>
+        <v>14700</v>
       </c>
       <c r="P50" s="7" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="Q50" s="7" t="n">
-        <v>3656</v>
+        <v>12216</v>
       </c>
       <c r="R50" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="S50" s="7" t="n">
-        <v>629273</v>
+        <v>0</v>
       </c>
       <c r="T50" s="5" t="n">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="U50" s="5" t="n">
-        <v>958770</v>
+        <v>426251</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>hemo</t>
+          <t>glucose_bld</t>
         </is>
       </c>
       <c r="B51" s="7" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="C51" s="7" t="n">
-        <v>64879</v>
+        <v>211779</v>
       </c>
       <c r="D51" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E51" s="7" t="n">
-        <v>3582</v>
+        <v>6763</v>
       </c>
       <c r="F51" s="7" t="n">
         <v>7</v>
       </c>
       <c r="G51" s="7" t="n">
-        <v>25115</v>
+        <v>25155</v>
       </c>
       <c r="H51" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I51" s="7" t="n">
-        <v>53674</v>
+        <v>0</v>
       </c>
       <c r="J51" s="7" t="n">
-        <v>18</v>
+        <v>102</v>
       </c>
       <c r="K51" s="7" t="n">
-        <v>102103</v>
+        <v>292594</v>
       </c>
       <c r="L51" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M51" s="7" t="n">
-        <v>23567</v>
+        <v>0</v>
       </c>
       <c r="N51" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O51" s="7" t="n">
-        <v>3746</v>
+        <v>10187</v>
       </c>
       <c r="P51" s="7" t="n">
         <v>2</v>
       </c>
       <c r="Q51" s="7" t="n">
-        <v>3655</v>
+        <v>358</v>
       </c>
       <c r="R51" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S51" s="7" t="n">
-        <v>629314</v>
+        <v>46598</v>
       </c>
       <c r="T51" s="5" t="n">
-        <v>46</v>
+        <v>139</v>
       </c>
       <c r="U51" s="5" t="n">
-        <v>909635</v>
+        <v>593434</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>hemo_a1c</t>
+          <t>hdl</t>
         </is>
       </c>
       <c r="B52" s="7" t="n">
-        <v>2</v>
+        <v>28</v>
       </c>
       <c r="C52" s="7" t="n">
-        <v>8841</v>
+        <v>282573</v>
       </c>
       <c r="D52" s="7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E52" s="7" t="n">
-        <v>0</v>
+        <v>16570</v>
       </c>
       <c r="F52" s="7" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G52" s="7" t="n">
-        <v>0</v>
+        <v>29869</v>
       </c>
       <c r="H52" s="7" t="n">
         <v>0</v>
@@ -4015,199 +4015,199 @@
         <v>0</v>
       </c>
       <c r="J52" s="7" t="n">
-        <v>9</v>
+        <v>52</v>
       </c>
       <c r="K52" s="7" t="n">
-        <v>55340</v>
+        <v>148153</v>
       </c>
       <c r="L52" s="7" t="n">
         <v>2</v>
       </c>
       <c r="M52" s="7" t="n">
-        <v>23612</v>
+        <v>23652</v>
       </c>
       <c r="N52" s="7" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="O52" s="7" t="n">
-        <v>28547</v>
+        <v>32797</v>
       </c>
       <c r="P52" s="7" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="Q52" s="7" t="n">
-        <v>20878</v>
+        <v>74205</v>
       </c>
       <c r="R52" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S52" s="7" t="n">
-        <v>0</v>
+        <v>46573</v>
       </c>
       <c r="T52" s="5" t="n">
-        <v>30</v>
+        <v>131</v>
       </c>
       <c r="U52" s="5" t="n">
-        <v>137218</v>
+        <v>654392</v>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>hip_circ</t>
+          <t>hemat</t>
         </is>
       </c>
       <c r="B53" s="7" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C53" s="7" t="n">
-        <v>54020</v>
+        <v>61658</v>
       </c>
       <c r="D53" s="7" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E53" s="7" t="n">
-        <v>33281</v>
+        <v>3582</v>
       </c>
       <c r="F53" s="7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G53" s="7" t="n">
-        <v>30339</v>
+        <v>25115</v>
       </c>
       <c r="H53" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>0</v>
+        <v>53674</v>
       </c>
       <c r="J53" s="7" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="K53" s="7" t="n">
-        <v>126492</v>
+        <v>154499</v>
       </c>
       <c r="L53" s="7" t="n">
         <v>2</v>
       </c>
       <c r="M53" s="7" t="n">
-        <v>23627</v>
+        <v>23567</v>
       </c>
       <c r="N53" s="7" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="O53" s="7" t="n">
-        <v>17671</v>
+        <v>3746</v>
       </c>
       <c r="P53" s="7" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="Q53" s="7" t="n">
-        <v>56541</v>
+        <v>3656</v>
       </c>
       <c r="R53" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S53" s="7" t="n">
-        <v>1610762</v>
+        <v>629273</v>
       </c>
       <c r="T53" s="5" t="n">
-        <v>84</v>
+        <v>67</v>
       </c>
       <c r="U53" s="5" t="n">
-        <v>1952733</v>
+        <v>958770</v>
       </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>hrtrt</t>
+          <t>hemo</t>
         </is>
       </c>
       <c r="B54" s="7" t="n">
-        <v>48</v>
+        <v>8</v>
       </c>
       <c r="C54" s="7" t="n">
-        <v>439669</v>
+        <v>64879</v>
       </c>
       <c r="D54" s="7" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E54" s="7" t="n">
-        <v>60109</v>
+        <v>3582</v>
       </c>
       <c r="F54" s="7" t="n">
-        <v>87</v>
+        <v>7</v>
       </c>
       <c r="G54" s="7" t="n">
-        <v>252223</v>
+        <v>25115</v>
       </c>
       <c r="H54" s="7" t="n">
         <v>3</v>
       </c>
       <c r="I54" s="7" t="n">
-        <v>64245</v>
+        <v>53674</v>
       </c>
       <c r="J54" s="7" t="n">
-        <v>62</v>
+        <v>18</v>
       </c>
       <c r="K54" s="7" t="n">
-        <v>185296</v>
+        <v>102103</v>
       </c>
       <c r="L54" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M54" s="7" t="n">
-        <v>35266</v>
+        <v>23567</v>
       </c>
       <c r="N54" s="7" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="O54" s="7" t="n">
-        <v>35238</v>
+        <v>3746</v>
       </c>
       <c r="P54" s="7" t="n">
-        <v>48</v>
+        <v>2</v>
       </c>
       <c r="Q54" s="7" t="n">
-        <v>154242</v>
+        <v>3655</v>
       </c>
       <c r="R54" s="7" t="n">
         <v>4</v>
       </c>
       <c r="S54" s="7" t="n">
-        <v>506519</v>
+        <v>629314</v>
       </c>
       <c r="T54" s="5" t="n">
-        <v>291</v>
+        <v>46</v>
       </c>
       <c r="U54" s="5" t="n">
-        <v>1732807</v>
+        <v>909635</v>
       </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>icam</t>
+          <t>hemo_a1c</t>
         </is>
       </c>
       <c r="B55" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C55" s="7" t="n">
-        <v>0</v>
+        <v>8841</v>
       </c>
       <c r="D55" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E55" s="7" t="n">
-        <v>2669</v>
+        <v>0</v>
       </c>
       <c r="F55" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G55" s="7" t="n">
-        <v>7663</v>
+        <v>0</v>
       </c>
       <c r="H55" s="7" t="n">
         <v>0</v>
@@ -4216,28 +4216,28 @@
         <v>0</v>
       </c>
       <c r="J55" s="7" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="K55" s="7" t="n">
-        <v>0</v>
+        <v>55340</v>
       </c>
       <c r="L55" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M55" s="7" t="n">
-        <v>0</v>
+        <v>23612</v>
       </c>
       <c r="N55" s="7" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="O55" s="7" t="n">
-        <v>0</v>
+        <v>28547</v>
       </c>
       <c r="P55" s="7" t="n">
         <v>6</v>
       </c>
       <c r="Q55" s="7" t="n">
-        <v>15379</v>
+        <v>20878</v>
       </c>
       <c r="R55" s="7" t="n">
         <v>0</v>
@@ -4246,35 +4246,35 @@
         <v>0</v>
       </c>
       <c r="T55" s="5" t="n">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="U55" s="5" t="n">
-        <v>25711</v>
+        <v>137218</v>
       </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>il10</t>
+          <t>hip_circ</t>
         </is>
       </c>
       <c r="B56" s="7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C56" s="7" t="n">
-        <v>0</v>
+        <v>54020</v>
       </c>
       <c r="D56" s="7" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E56" s="7" t="n">
-        <v>0</v>
+        <v>33281</v>
       </c>
       <c r="F56" s="7" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G56" s="7" t="n">
-        <v>0</v>
+        <v>30339</v>
       </c>
       <c r="H56" s="7" t="n">
         <v>0</v>
@@ -4283,113 +4283,113 @@
         <v>0</v>
       </c>
       <c r="J56" s="7" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="K56" s="7" t="n">
-        <v>0</v>
+        <v>126492</v>
       </c>
       <c r="L56" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M56" s="7" t="n">
-        <v>0</v>
+        <v>23627</v>
       </c>
       <c r="N56" s="7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="O56" s="7" t="n">
-        <v>0</v>
+        <v>17671</v>
       </c>
       <c r="P56" s="7" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="Q56" s="7" t="n">
-        <v>943</v>
+        <v>56541</v>
       </c>
       <c r="R56" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S56" s="7" t="n">
-        <v>0</v>
+        <v>1610762</v>
       </c>
       <c r="T56" s="5" t="n">
-        <v>2</v>
+        <v>84</v>
       </c>
       <c r="U56" s="5" t="n">
-        <v>943</v>
+        <v>1952733</v>
       </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>il18</t>
+          <t>hrtrt</t>
         </is>
       </c>
       <c r="B57" s="7" t="n">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="C57" s="7" t="n">
-        <v>0</v>
+        <v>439669</v>
       </c>
       <c r="D57" s="7" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="E57" s="7" t="n">
-        <v>0</v>
+        <v>60109</v>
       </c>
       <c r="F57" s="7" t="n">
-        <v>0</v>
+        <v>87</v>
       </c>
       <c r="G57" s="7" t="n">
-        <v>0</v>
+        <v>252223</v>
       </c>
       <c r="H57" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>0</v>
+        <v>64245</v>
       </c>
       <c r="J57" s="7" t="n">
+        <v>62</v>
+      </c>
+      <c r="K57" s="7" t="n">
+        <v>185296</v>
+      </c>
+      <c r="L57" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="M57" s="7" t="n">
+        <v>35266</v>
+      </c>
+      <c r="N57" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="O57" s="7" t="n">
+        <v>35238</v>
+      </c>
+      <c r="P57" s="7" t="n">
+        <v>48</v>
+      </c>
+      <c r="Q57" s="7" t="n">
+        <v>154242</v>
+      </c>
+      <c r="R57" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="K57" s="7" t="n">
-        <v>38307</v>
-      </c>
-      <c r="L57" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M57" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N57" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O57" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P57" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q57" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="R57" s="7" t="n">
-        <v>0</v>
-      </c>
       <c r="S57" s="7" t="n">
-        <v>0</v>
+        <v>506519</v>
       </c>
       <c r="T57" s="5" t="n">
-        <v>4</v>
+        <v>291</v>
       </c>
       <c r="U57" s="5" t="n">
-        <v>38307</v>
+        <v>1732807</v>
       </c>
     </row>
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>il6</t>
+          <t>icam</t>
         </is>
       </c>
       <c r="B58" s="7" t="n">
@@ -4402,13 +4402,13 @@
         <v>1</v>
       </c>
       <c r="E58" s="7" t="n">
-        <v>689</v>
+        <v>2669</v>
       </c>
       <c r="F58" s="7" t="n">
         <v>2</v>
       </c>
       <c r="G58" s="7" t="n">
-        <v>10594</v>
+        <v>7663</v>
       </c>
       <c r="H58" s="7" t="n">
         <v>0</v>
@@ -4438,7 +4438,7 @@
         <v>6</v>
       </c>
       <c r="Q58" s="7" t="n">
-        <v>17277</v>
+        <v>15379</v>
       </c>
       <c r="R58" s="7" t="n">
         <v>0</v>
@@ -4450,32 +4450,32 @@
         <v>9</v>
       </c>
       <c r="U58" s="5" t="n">
-        <v>28560</v>
+        <v>25711</v>
       </c>
     </row>
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>insulin_blood</t>
+          <t>il10</t>
         </is>
       </c>
       <c r="B59" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C59" s="7" t="n">
-        <v>56942</v>
+        <v>0</v>
       </c>
       <c r="D59" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E59" s="7" t="n">
-        <v>9647</v>
+        <v>0</v>
       </c>
       <c r="F59" s="7" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G59" s="7" t="n">
-        <v>25071</v>
+        <v>0</v>
       </c>
       <c r="H59" s="7" t="n">
         <v>0</v>
@@ -4484,46 +4484,46 @@
         <v>0</v>
       </c>
       <c r="J59" s="7" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="K59" s="7" t="n">
-        <v>74472</v>
+        <v>0</v>
       </c>
       <c r="L59" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M59" s="7" t="n">
-        <v>23618</v>
+        <v>0</v>
       </c>
       <c r="N59" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O59" s="7" t="n">
-        <v>6587</v>
+        <v>0</v>
       </c>
       <c r="P59" s="7" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="Q59" s="7" t="n">
-        <v>25329</v>
+        <v>943</v>
       </c>
       <c r="R59" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S59" s="7" t="n">
-        <v>43342</v>
+        <v>0</v>
       </c>
       <c r="T59" s="5" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="U59" s="5" t="n">
-        <v>265008</v>
+        <v>943</v>
       </c>
     </row>
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>isoprostane_8_epi_pgf2a</t>
+          <t>il18</t>
         </is>
       </c>
       <c r="B60" s="7" t="n">
@@ -4533,10 +4533,10 @@
         <v>0</v>
       </c>
       <c r="D60" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E60" s="7" t="n">
-        <v>2720</v>
+        <v>0</v>
       </c>
       <c r="F60" s="7" t="n">
         <v>0</v>
@@ -4551,10 +4551,10 @@
         <v>0</v>
       </c>
       <c r="J60" s="7" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K60" s="7" t="n">
-        <v>0</v>
+        <v>38307</v>
       </c>
       <c r="L60" s="7" t="n">
         <v>0</v>
@@ -4569,10 +4569,10 @@
         <v>0</v>
       </c>
       <c r="P60" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q60" s="7" t="n">
-        <v>6805</v>
+        <v>0</v>
       </c>
       <c r="R60" s="7" t="n">
         <v>0</v>
@@ -4581,16 +4581,16 @@
         <v>0</v>
       </c>
       <c r="T60" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U60" s="5" t="n">
-        <v>9525</v>
+        <v>38307</v>
       </c>
     </row>
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>lactate</t>
+          <t>il6</t>
         </is>
       </c>
       <c r="B61" s="7" t="n">
@@ -4600,16 +4600,16 @@
         <v>0</v>
       </c>
       <c r="D61" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E61" s="7" t="n">
-        <v>0</v>
+        <v>689</v>
       </c>
       <c r="F61" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G61" s="7" t="n">
-        <v>0</v>
+        <v>10594</v>
       </c>
       <c r="H61" s="7" t="n">
         <v>0</v>
@@ -4618,10 +4618,10 @@
         <v>0</v>
       </c>
       <c r="J61" s="7" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K61" s="7" t="n">
-        <v>26148</v>
+        <v>0</v>
       </c>
       <c r="L61" s="7" t="n">
         <v>0</v>
@@ -4636,10 +4636,10 @@
         <v>0</v>
       </c>
       <c r="P61" s="7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Q61" s="7" t="n">
-        <v>0</v>
+        <v>17277</v>
       </c>
       <c r="R61" s="7" t="n">
         <v>0</v>
@@ -4648,35 +4648,35 @@
         <v>0</v>
       </c>
       <c r="T61" s="5" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="U61" s="5" t="n">
-        <v>26148</v>
+        <v>28560</v>
       </c>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>lactate_dehyd</t>
+          <t>insulin_blood</t>
         </is>
       </c>
       <c r="B62" s="7" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C62" s="7" t="n">
-        <v>0</v>
+        <v>56942</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E62" s="7" t="n">
-        <v>0</v>
+        <v>9647</v>
       </c>
       <c r="F62" s="7" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>0</v>
+        <v>25071</v>
       </c>
       <c r="H62" s="7" t="n">
         <v>0</v>
@@ -4685,65 +4685,65 @@
         <v>0</v>
       </c>
       <c r="J62" s="7" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="K62" s="7" t="n">
-        <v>3530</v>
+        <v>74472</v>
       </c>
       <c r="L62" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M62" s="7" t="n">
-        <v>0</v>
+        <v>23618</v>
       </c>
       <c r="N62" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O62" s="7" t="n">
-        <v>0</v>
+        <v>6587</v>
       </c>
       <c r="P62" s="7" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="Q62" s="7" t="n">
-        <v>0</v>
+        <v>25329</v>
       </c>
       <c r="R62" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S62" s="7" t="n">
-        <v>0</v>
+        <v>43342</v>
       </c>
       <c r="T62" s="5" t="n">
-        <v>3</v>
+        <v>41</v>
       </c>
       <c r="U62" s="5" t="n">
-        <v>3530</v>
+        <v>265008</v>
       </c>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>ldl</t>
+          <t>isoprostane_8_epi_pgf2a</t>
         </is>
       </c>
       <c r="B63" s="7" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="C63" s="7" t="n">
-        <v>173272</v>
+        <v>0</v>
       </c>
       <c r="D63" s="7" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E63" s="7" t="n">
-        <v>16477</v>
+        <v>2720</v>
       </c>
       <c r="F63" s="7" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G63" s="7" t="n">
-        <v>25015</v>
+        <v>0</v>
       </c>
       <c r="H63" s="7" t="n">
         <v>0</v>
@@ -4752,46 +4752,46 @@
         <v>0</v>
       </c>
       <c r="J63" s="7" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="K63" s="7" t="n">
-        <v>123639</v>
+        <v>0</v>
       </c>
       <c r="L63" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M63" s="7" t="n">
-        <v>23409</v>
+        <v>0</v>
       </c>
       <c r="N63" s="7" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="O63" s="7" t="n">
-        <v>43886</v>
+        <v>0</v>
       </c>
       <c r="P63" s="7" t="n">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="Q63" s="7" t="n">
-        <v>68027</v>
+        <v>6805</v>
       </c>
       <c r="R63" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S63" s="7" t="n">
-        <v>46331</v>
+        <v>0</v>
       </c>
       <c r="T63" s="5" t="n">
-        <v>112</v>
+        <v>3</v>
       </c>
       <c r="U63" s="5" t="n">
-        <v>520056</v>
+        <v>9525</v>
       </c>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>lppla2_act</t>
+          <t>lactate</t>
         </is>
       </c>
       <c r="B64" s="7" t="n">
@@ -4807,10 +4807,10 @@
         <v>0</v>
       </c>
       <c r="F64" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>10910</v>
+        <v>0</v>
       </c>
       <c r="H64" s="7" t="n">
         <v>0</v>
@@ -4819,10 +4819,10 @@
         <v>0</v>
       </c>
       <c r="J64" s="7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="K64" s="7" t="n">
-        <v>0</v>
+        <v>26148</v>
       </c>
       <c r="L64" s="7" t="n">
         <v>0</v>
@@ -4837,10 +4837,10 @@
         <v>0</v>
       </c>
       <c r="P64" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q64" s="7" t="n">
-        <v>5122</v>
+        <v>0</v>
       </c>
       <c r="R64" s="7" t="n">
         <v>0</v>
@@ -4849,16 +4849,16 @@
         <v>0</v>
       </c>
       <c r="T64" s="5" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="U64" s="5" t="n">
-        <v>16032</v>
+        <v>26148</v>
       </c>
     </row>
     <row r="65" ht="18" customHeight="1">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>lppla2_mass</t>
+          <t>lactate_dehyd</t>
         </is>
       </c>
       <c r="B65" s="7" t="n">
@@ -4874,10 +4874,10 @@
         <v>0</v>
       </c>
       <c r="F65" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G65" s="7" t="n">
-        <v>10923</v>
+        <v>0</v>
       </c>
       <c r="H65" s="7" t="n">
         <v>0</v>
@@ -4886,10 +4886,10 @@
         <v>0</v>
       </c>
       <c r="J65" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K65" s="7" t="n">
-        <v>0</v>
+        <v>3530</v>
       </c>
       <c r="L65" s="7" t="n">
         <v>0</v>
@@ -4904,10 +4904,10 @@
         <v>0</v>
       </c>
       <c r="P65" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q65" s="7" t="n">
-        <v>5042</v>
+        <v>0</v>
       </c>
       <c r="R65" s="7" t="n">
         <v>0</v>
@@ -4919,87 +4919,87 @@
         <v>3</v>
       </c>
       <c r="U65" s="5" t="n">
-        <v>15965</v>
+        <v>3530</v>
       </c>
     </row>
     <row r="66" ht="18" customHeight="1">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>lympho_ct</t>
+          <t>ldl</t>
         </is>
       </c>
       <c r="B66" s="7" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>5706</v>
+        <v>173272</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E66" s="7" t="n">
-        <v>3968</v>
+        <v>16477</v>
       </c>
       <c r="F66" s="7" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>0</v>
+        <v>25015</v>
       </c>
       <c r="H66" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I66" s="7" t="n">
-        <v>53590</v>
+        <v>0</v>
       </c>
       <c r="J66" s="7" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="K66" s="7" t="n">
-        <v>0</v>
+        <v>123639</v>
       </c>
       <c r="L66" s="7" t="n">
         <v>2</v>
       </c>
       <c r="M66" s="7" t="n">
-        <v>22908</v>
+        <v>23409</v>
       </c>
       <c r="N66" s="7" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="O66" s="7" t="n">
-        <v>0</v>
+        <v>43886</v>
       </c>
       <c r="P66" s="7" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="Q66" s="7" t="n">
-        <v>2338</v>
+        <v>68027</v>
       </c>
       <c r="R66" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S66" s="7" t="n">
-        <v>0</v>
+        <v>46331</v>
       </c>
       <c r="T66" s="5" t="n">
-        <v>10</v>
+        <v>112</v>
       </c>
       <c r="U66" s="5" t="n">
-        <v>88510</v>
+        <v>520056</v>
       </c>
     </row>
     <row r="67" ht="18" customHeight="1">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>lympho_pct</t>
+          <t>lppla2_act</t>
         </is>
       </c>
       <c r="B67" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C67" s="7" t="n">
-        <v>24362</v>
+        <v>0</v>
       </c>
       <c r="D67" s="7" t="n">
         <v>0</v>
@@ -5008,10 +5008,10 @@
         <v>0</v>
       </c>
       <c r="F67" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G67" s="7" t="n">
-        <v>0</v>
+        <v>10910</v>
       </c>
       <c r="H67" s="7" t="n">
         <v>0</v>
@@ -5020,28 +5020,28 @@
         <v>0</v>
       </c>
       <c r="J67" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K67" s="7" t="n">
-        <v>12638</v>
+        <v>0</v>
       </c>
       <c r="L67" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M67" s="7" t="n">
-        <v>22908</v>
+        <v>0</v>
       </c>
       <c r="N67" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O67" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P67" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="O67" s="7" t="n">
-        <v>3362</v>
-      </c>
-      <c r="P67" s="7" t="n">
-        <v>0</v>
-      </c>
       <c r="Q67" s="7" t="n">
-        <v>0</v>
+        <v>5122</v>
       </c>
       <c r="R67" s="7" t="n">
         <v>0</v>
@@ -5050,65 +5050,65 @@
         <v>0</v>
       </c>
       <c r="T67" s="5" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="U67" s="5" t="n">
-        <v>63270</v>
+        <v>16032</v>
       </c>
     </row>
     <row r="68" ht="18" customHeight="1">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>mch</t>
+          <t>lppla2_mass</t>
         </is>
       </c>
       <c r="B68" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C68" s="7" t="n">
-        <v>12069</v>
+        <v>0</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E68" s="7" t="n">
-        <v>7165</v>
+        <v>0</v>
       </c>
       <c r="F68" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G68" s="7" t="n">
-        <v>0</v>
+        <v>10923</v>
       </c>
       <c r="H68" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I68" s="7" t="n">
-        <v>53674</v>
+        <v>0</v>
       </c>
       <c r="J68" s="7" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="K68" s="7" t="n">
-        <v>54003</v>
+        <v>0</v>
       </c>
       <c r="L68" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M68" s="7" t="n">
-        <v>23567</v>
+        <v>0</v>
       </c>
       <c r="N68" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O68" s="7" t="n">
-        <v>3376</v>
+        <v>0</v>
       </c>
       <c r="P68" s="7" t="n">
         <v>1</v>
       </c>
       <c r="Q68" s="7" t="n">
-        <v>2756</v>
+        <v>5042</v>
       </c>
       <c r="R68" s="7" t="n">
         <v>0</v>
@@ -5117,29 +5117,29 @@
         <v>0</v>
       </c>
       <c r="T68" s="5" t="n">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="U68" s="5" t="n">
-        <v>156610</v>
+        <v>15965</v>
       </c>
     </row>
     <row r="69" ht="18" customHeight="1">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>mchc</t>
+          <t>lympho_ct</t>
         </is>
       </c>
       <c r="B69" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C69" s="7" t="n">
-        <v>8408</v>
+        <v>5706</v>
       </c>
       <c r="D69" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E69" s="7" t="n">
-        <v>0</v>
+        <v>3968</v>
       </c>
       <c r="F69" s="7" t="n">
         <v>0</v>
@@ -5151,31 +5151,31 @@
         <v>3</v>
       </c>
       <c r="I69" s="7" t="n">
-        <v>53674</v>
+        <v>53590</v>
       </c>
       <c r="J69" s="7" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="K69" s="7" t="n">
-        <v>39615</v>
+        <v>0</v>
       </c>
       <c r="L69" s="7" t="n">
         <v>2</v>
       </c>
       <c r="M69" s="7" t="n">
-        <v>23567</v>
+        <v>22908</v>
       </c>
       <c r="N69" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O69" s="7" t="n">
-        <v>3377</v>
+        <v>0</v>
       </c>
       <c r="P69" s="7" t="n">
         <v>1</v>
       </c>
       <c r="Q69" s="7" t="n">
-        <v>2756</v>
+        <v>2338</v>
       </c>
       <c r="R69" s="7" t="n">
         <v>0</v>
@@ -5184,23 +5184,23 @@
         <v>0</v>
       </c>
       <c r="T69" s="5" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="U69" s="5" t="n">
-        <v>131397</v>
+        <v>88510</v>
       </c>
     </row>
     <row r="70" ht="18" customHeight="1">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>mcv</t>
+          <t>lympho_pct</t>
         </is>
       </c>
       <c r="B70" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>28238</v>
+        <v>24362</v>
       </c>
       <c r="D70" s="7" t="n">
         <v>0</v>
@@ -5215,34 +5215,34 @@
         <v>0</v>
       </c>
       <c r="H70" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I70" s="7" t="n">
-        <v>53674</v>
+        <v>0</v>
       </c>
       <c r="J70" s="7" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="K70" s="7" t="n">
-        <v>39615</v>
+        <v>12638</v>
       </c>
       <c r="L70" s="7" t="n">
         <v>2</v>
       </c>
       <c r="M70" s="7" t="n">
-        <v>23567</v>
+        <v>22908</v>
       </c>
       <c r="N70" s="7" t="n">
         <v>1</v>
       </c>
       <c r="O70" s="7" t="n">
-        <v>3377</v>
+        <v>3362</v>
       </c>
       <c r="P70" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q70" s="7" t="n">
-        <v>2756</v>
+        <v>0</v>
       </c>
       <c r="R70" s="7" t="n">
         <v>0</v>
@@ -5251,29 +5251,29 @@
         <v>0</v>
       </c>
       <c r="T70" s="5" t="n">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="U70" s="5" t="n">
-        <v>151227</v>
+        <v>63270</v>
       </c>
     </row>
     <row r="71" ht="18" customHeight="1">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>mean_art_press</t>
+          <t>mch</t>
         </is>
       </c>
       <c r="B71" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C71" s="7" t="n">
-        <v>0</v>
+        <v>12069</v>
       </c>
       <c r="D71" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E71" s="7" t="n">
-        <v>0</v>
+        <v>7165</v>
       </c>
       <c r="F71" s="7" t="n">
         <v>0</v>
@@ -5282,34 +5282,34 @@
         <v>0</v>
       </c>
       <c r="H71" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I71" s="7" t="n">
-        <v>0</v>
+        <v>53674</v>
       </c>
       <c r="J71" s="7" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="K71" s="7" t="n">
-        <v>50002</v>
+        <v>54003</v>
       </c>
       <c r="L71" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M71" s="7" t="n">
-        <v>0</v>
+        <v>23567</v>
       </c>
       <c r="N71" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O71" s="7" t="n">
-        <v>0</v>
+        <v>3376</v>
       </c>
       <c r="P71" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q71" s="7" t="n">
-        <v>0</v>
+        <v>2756</v>
       </c>
       <c r="R71" s="7" t="n">
         <v>0</v>
@@ -5318,23 +5318,23 @@
         <v>0</v>
       </c>
       <c r="T71" s="5" t="n">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="U71" s="5" t="n">
-        <v>50002</v>
+        <v>156610</v>
       </c>
     </row>
     <row r="72" ht="18" customHeight="1">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>mmp9</t>
+          <t>mchc</t>
         </is>
       </c>
       <c r="B72" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>0</v>
+        <v>8408</v>
       </c>
       <c r="D72" s="7" t="n">
         <v>0</v>
@@ -5349,34 +5349,34 @@
         <v>0</v>
       </c>
       <c r="H72" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I72" s="7" t="n">
-        <v>0</v>
+        <v>53674</v>
       </c>
       <c r="J72" s="7" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="K72" s="7" t="n">
-        <v>0</v>
+        <v>39615</v>
       </c>
       <c r="L72" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M72" s="7" t="n">
-        <v>0</v>
+        <v>23567</v>
       </c>
       <c r="N72" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O72" s="7" t="n">
-        <v>0</v>
+        <v>3377</v>
       </c>
       <c r="P72" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q72" s="7" t="n">
-        <v>7393</v>
+        <v>2756</v>
       </c>
       <c r="R72" s="7" t="n">
         <v>0</v>
@@ -5385,65 +5385,65 @@
         <v>0</v>
       </c>
       <c r="T72" s="5" t="n">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="U72" s="5" t="n">
-        <v>7393</v>
+        <v>131397</v>
       </c>
     </row>
     <row r="73" ht="18" customHeight="1">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>mn_art_pres</t>
+          <t>mcv</t>
         </is>
       </c>
       <c r="B73" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C73" s="7" t="n">
+        <v>28238</v>
+      </c>
+      <c r="D73" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E73" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F73" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G73" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H73" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="I73" s="7" t="n">
+        <v>53674</v>
+      </c>
+      <c r="J73" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="K73" s="7" t="n">
+        <v>39615</v>
+      </c>
+      <c r="L73" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="M73" s="7" t="n">
+        <v>23567</v>
+      </c>
+      <c r="N73" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="C73" s="7" t="n">
-        <v>18</v>
-      </c>
-      <c r="D73" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E73" s="7" t="n">
-        <v>24769</v>
-      </c>
-      <c r="F73" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G73" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H73" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I73" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J73" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K73" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L73" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M73" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N73" s="7" t="n">
-        <v>0</v>
-      </c>
       <c r="O73" s="7" t="n">
-        <v>0</v>
+        <v>3377</v>
       </c>
       <c r="P73" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q73" s="7" t="n">
-        <v>18383</v>
+        <v>2756</v>
       </c>
       <c r="R73" s="7" t="n">
         <v>0</v>
@@ -5452,29 +5452,29 @@
         <v>0</v>
       </c>
       <c r="T73" s="5" t="n">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="U73" s="5" t="n">
-        <v>43170</v>
+        <v>151227</v>
       </c>
     </row>
     <row r="74" ht="18" customHeight="1">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>monocyte_ncnc_bld</t>
+          <t>mean_art_press</t>
         </is>
       </c>
       <c r="B74" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C74" s="7" t="n">
-        <v>5706</v>
+        <v>0</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E74" s="7" t="n">
-        <v>384</v>
+        <v>0</v>
       </c>
       <c r="F74" s="7" t="n">
         <v>0</v>
@@ -5483,22 +5483,22 @@
         <v>0</v>
       </c>
       <c r="H74" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I74" s="7" t="n">
-        <v>53588</v>
+        <v>0</v>
       </c>
       <c r="J74" s="7" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="K74" s="7" t="n">
-        <v>32540</v>
+        <v>50002</v>
       </c>
       <c r="L74" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M74" s="7" t="n">
-        <v>22913</v>
+        <v>0</v>
       </c>
       <c r="N74" s="7" t="n">
         <v>0</v>
@@ -5507,10 +5507,10 @@
         <v>0</v>
       </c>
       <c r="P74" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q74" s="7" t="n">
-        <v>3231</v>
+        <v>0</v>
       </c>
       <c r="R74" s="7" t="n">
         <v>0</v>
@@ -5519,29 +5519,29 @@
         <v>0</v>
       </c>
       <c r="T74" s="5" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="U74" s="5" t="n">
-        <v>118362</v>
+        <v>50002</v>
       </c>
     </row>
     <row r="75" ht="18" customHeight="1">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>neutro_pct</t>
+          <t>mmp9</t>
         </is>
       </c>
       <c r="B75" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C75" s="7" t="n">
-        <v>18618</v>
+        <v>0</v>
       </c>
       <c r="D75" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E75" s="7" t="n">
-        <v>2407</v>
+        <v>0</v>
       </c>
       <c r="F75" s="7" t="n">
         <v>0</v>
@@ -5562,10 +5562,10 @@
         <v>0</v>
       </c>
       <c r="L75" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M75" s="7" t="n">
-        <v>22908</v>
+        <v>0</v>
       </c>
       <c r="N75" s="7" t="n">
         <v>0</v>
@@ -5574,10 +5574,10 @@
         <v>0</v>
       </c>
       <c r="P75" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q75" s="7" t="n">
-        <v>0</v>
+        <v>7393</v>
       </c>
       <c r="R75" s="7" t="n">
         <v>0</v>
@@ -5586,29 +5586,29 @@
         <v>0</v>
       </c>
       <c r="T75" s="5" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="U75" s="5" t="n">
-        <v>43933</v>
+        <v>7393</v>
       </c>
     </row>
     <row r="76" ht="18" customHeight="1">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>neutrophil_ct</t>
+          <t>mn_art_pres</t>
         </is>
       </c>
       <c r="B76" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C76" s="7" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="D76" s="7" t="n">
         <v>2</v>
       </c>
       <c r="E76" s="7" t="n">
-        <v>324</v>
+        <v>24769</v>
       </c>
       <c r="F76" s="7" t="n">
         <v>0</v>
@@ -5617,10 +5617,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I76" s="7" t="n">
-        <v>53590</v>
+        <v>0</v>
       </c>
       <c r="J76" s="7" t="n">
         <v>0</v>
@@ -5629,10 +5629,10 @@
         <v>0</v>
       </c>
       <c r="L76" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M76" s="7" t="n">
-        <v>22909</v>
+        <v>0</v>
       </c>
       <c r="N76" s="7" t="n">
         <v>0</v>
@@ -5641,10 +5641,10 @@
         <v>0</v>
       </c>
       <c r="P76" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q76" s="7" t="n">
-        <v>2338</v>
+        <v>18383</v>
       </c>
       <c r="R76" s="7" t="n">
         <v>0</v>
@@ -5653,29 +5653,29 @@
         <v>0</v>
       </c>
       <c r="T76" s="5" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="U76" s="5" t="n">
-        <v>79161</v>
+        <v>43170</v>
       </c>
     </row>
     <row r="77" ht="18" customHeight="1">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>nt_bnp</t>
+          <t>monocyte_ncnc_bld</t>
         </is>
       </c>
       <c r="B77" s="7" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="C77" s="7" t="n">
-        <v>47302</v>
+        <v>5706</v>
       </c>
       <c r="D77" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E77" s="7" t="n">
-        <v>0</v>
+        <v>384</v>
       </c>
       <c r="F77" s="7" t="n">
         <v>0</v>
@@ -5684,22 +5684,22 @@
         <v>0</v>
       </c>
       <c r="H77" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I77" s="7" t="n">
-        <v>0</v>
+        <v>53588</v>
       </c>
       <c r="J77" s="7" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K77" s="7" t="n">
-        <v>19114</v>
+        <v>32540</v>
       </c>
       <c r="L77" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M77" s="7" t="n">
-        <v>0</v>
+        <v>22913</v>
       </c>
       <c r="N77" s="7" t="n">
         <v>0</v>
@@ -5711,38 +5711,38 @@
         <v>2</v>
       </c>
       <c r="Q77" s="7" t="n">
-        <v>10090</v>
+        <v>3231</v>
       </c>
       <c r="R77" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S77" s="7" t="n">
-        <v>1802</v>
+        <v>0</v>
       </c>
       <c r="T77" s="5" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="U77" s="5" t="n">
-        <v>78308</v>
+        <v>118362</v>
       </c>
     </row>
     <row r="78" ht="18" customHeight="1">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>pacem_stat</t>
+          <t>neutro_pct</t>
         </is>
       </c>
       <c r="B78" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C78" s="7" t="n">
-        <v>13110</v>
+        <v>18618</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E78" s="7" t="n">
-        <v>0</v>
+        <v>2407</v>
       </c>
       <c r="F78" s="7" t="n">
         <v>0</v>
@@ -5766,7 +5766,7 @@
         <v>2</v>
       </c>
       <c r="M78" s="7" t="n">
-        <v>11848</v>
+        <v>22908</v>
       </c>
       <c r="N78" s="7" t="n">
         <v>0</v>
@@ -5775,10 +5775,10 @@
         <v>0</v>
       </c>
       <c r="P78" s="7" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="Q78" s="7" t="n">
-        <v>12922</v>
+        <v>0</v>
       </c>
       <c r="R78" s="7" t="n">
         <v>0</v>
@@ -5787,90 +5787,90 @@
         <v>0</v>
       </c>
       <c r="T78" s="5" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="U78" s="5" t="n">
-        <v>37880</v>
+        <v>43933</v>
       </c>
     </row>
     <row r="79" ht="18" customHeight="1">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>platelet_ct</t>
+          <t>neutrophil_ct</t>
         </is>
       </c>
       <c r="B79" s="7" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="C79" s="7" t="n">
-        <v>37442</v>
+        <v>0</v>
       </c>
       <c r="D79" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E79" s="7" t="n">
+        <v>324</v>
+      </c>
+      <c r="F79" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G79" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H79" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="I79" s="7" t="n">
+        <v>53590</v>
+      </c>
+      <c r="J79" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K79" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L79" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="M79" s="7" t="n">
+        <v>22909</v>
+      </c>
+      <c r="N79" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O79" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P79" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E79" s="7" t="n">
-        <v>3581</v>
-      </c>
-      <c r="F79" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="G79" s="7" t="n">
-        <v>25046</v>
-      </c>
-      <c r="H79" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="I79" s="7" t="n">
-        <v>53654</v>
-      </c>
-      <c r="J79" s="7" t="n">
+      <c r="Q79" s="7" t="n">
+        <v>2338</v>
+      </c>
+      <c r="R79" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S79" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T79" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="K79" s="7" t="n">
-        <v>35931</v>
-      </c>
-      <c r="L79" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="M79" s="7" t="n">
-        <v>23560</v>
-      </c>
-      <c r="N79" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="O79" s="7" t="n">
-        <v>3749</v>
-      </c>
-      <c r="P79" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q79" s="7" t="n">
-        <v>3644</v>
-      </c>
-      <c r="R79" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="S79" s="7" t="n">
-        <v>623065</v>
-      </c>
-      <c r="T79" s="5" t="n">
-        <v>33</v>
-      </c>
       <c r="U79" s="5" t="n">
-        <v>809672</v>
+        <v>79161</v>
       </c>
     </row>
     <row r="80" ht="18" customHeight="1">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>pmv</t>
+          <t>nt_bnp</t>
         </is>
       </c>
       <c r="B80" s="7" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="C80" s="7" t="n">
-        <v>5707</v>
+        <v>47302</v>
       </c>
       <c r="D80" s="7" t="n">
         <v>0</v>
@@ -5891,10 +5891,10 @@
         <v>0</v>
       </c>
       <c r="J80" s="7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K80" s="7" t="n">
-        <v>32540</v>
+        <v>19114</v>
       </c>
       <c r="L80" s="7" t="n">
         <v>0</v>
@@ -5903,53 +5903,53 @@
         <v>0</v>
       </c>
       <c r="N80" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O80" s="7" t="n">
-        <v>3376</v>
+        <v>0</v>
       </c>
       <c r="P80" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q80" s="7" t="n">
-        <v>0</v>
+        <v>10090</v>
       </c>
       <c r="R80" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S80" s="7" t="n">
-        <v>0</v>
+        <v>1802</v>
       </c>
       <c r="T80" s="5" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="U80" s="5" t="n">
-        <v>41623</v>
+        <v>78308</v>
       </c>
     </row>
     <row r="81" ht="18" customHeight="1">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>potassium</t>
+          <t>pacem_stat</t>
         </is>
       </c>
       <c r="B81" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C81" s="7" t="n">
-        <v>37384</v>
+        <v>13110</v>
       </c>
       <c r="D81" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E81" s="7" t="n">
-        <v>6310</v>
+        <v>0</v>
       </c>
       <c r="F81" s="7" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G81" s="7" t="n">
-        <v>25155</v>
+        <v>0</v>
       </c>
       <c r="H81" s="7" t="n">
         <v>0</v>
@@ -5964,22 +5964,22 @@
         <v>0</v>
       </c>
       <c r="L81" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M81" s="7" t="n">
-        <v>0</v>
+        <v>11848</v>
       </c>
       <c r="N81" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O81" s="7" t="n">
-        <v>3839</v>
+        <v>0</v>
       </c>
       <c r="P81" s="7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="Q81" s="7" t="n">
-        <v>18964</v>
+        <v>12922</v>
       </c>
       <c r="R81" s="7" t="n">
         <v>0</v>
@@ -5988,90 +5988,90 @@
         <v>0</v>
       </c>
       <c r="T81" s="5" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="U81" s="5" t="n">
-        <v>91652</v>
+        <v>37880</v>
       </c>
     </row>
     <row r="82" ht="18" customHeight="1">
       <c r="A82" s="6" t="inlineStr">
         <is>
-          <t>pr_ekg</t>
+          <t>platelet_ct</t>
         </is>
       </c>
       <c r="B82" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C82" s="7" t="n">
-        <v>59015</v>
+        <v>37442</v>
       </c>
       <c r="D82" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E82" s="7" t="n">
-        <v>0</v>
+        <v>3581</v>
       </c>
       <c r="F82" s="7" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G82" s="7" t="n">
-        <v>0</v>
+        <v>25046</v>
       </c>
       <c r="H82" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I82" s="7" t="n">
-        <v>0</v>
+        <v>53654</v>
       </c>
       <c r="J82" s="7" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="K82" s="7" t="n">
-        <v>0</v>
+        <v>35931</v>
       </c>
       <c r="L82" s="7" t="n">
         <v>2</v>
       </c>
       <c r="M82" s="7" t="n">
-        <v>23526</v>
+        <v>23560</v>
       </c>
       <c r="N82" s="7" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="O82" s="7" t="n">
-        <v>78673</v>
+        <v>3749</v>
       </c>
       <c r="P82" s="7" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="Q82" s="7" t="n">
-        <v>22435</v>
+        <v>3644</v>
       </c>
       <c r="R82" s="7" t="n">
         <v>3</v>
       </c>
       <c r="S82" s="7" t="n">
-        <v>500439</v>
+        <v>623065</v>
       </c>
       <c r="T82" s="5" t="n">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="U82" s="5" t="n">
-        <v>684088</v>
+        <v>809672</v>
       </c>
     </row>
     <row r="83" ht="18" customHeight="1">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>pr_qrs_qt</t>
+          <t>pmv</t>
         </is>
       </c>
       <c r="B83" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C83" s="7" t="n">
-        <v>0</v>
+        <v>5707</v>
       </c>
       <c r="D83" s="7" t="n">
         <v>0</v>
@@ -6092,10 +6092,10 @@
         <v>0</v>
       </c>
       <c r="J83" s="7" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K83" s="7" t="n">
-        <v>66296</v>
+        <v>32540</v>
       </c>
       <c r="L83" s="7" t="n">
         <v>0</v>
@@ -6104,10 +6104,10 @@
         <v>0</v>
       </c>
       <c r="N83" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O83" s="7" t="n">
-        <v>0</v>
+        <v>3376</v>
       </c>
       <c r="P83" s="7" t="n">
         <v>0</v>
@@ -6122,35 +6122,35 @@
         <v>0</v>
       </c>
       <c r="T83" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="U83" s="5" t="n">
-        <v>66296</v>
+        <v>41623</v>
       </c>
     </row>
     <row r="84" ht="18" customHeight="1">
       <c r="A84" s="6" t="inlineStr">
         <is>
-          <t>pselectin</t>
+          <t>potassium</t>
         </is>
       </c>
       <c r="B84" s="7" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C84" s="7" t="n">
-        <v>0</v>
+        <v>37384</v>
       </c>
       <c r="D84" s="7" t="n">
         <v>2</v>
       </c>
       <c r="E84" s="7" t="n">
-        <v>326</v>
+        <v>6310</v>
       </c>
       <c r="F84" s="7" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G84" s="7" t="n">
-        <v>0</v>
+        <v>25155</v>
       </c>
       <c r="H84" s="7" t="n">
         <v>0</v>
@@ -6171,16 +6171,16 @@
         <v>0</v>
       </c>
       <c r="N84" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O84" s="7" t="n">
-        <v>8299</v>
+        <v>3839</v>
       </c>
       <c r="P84" s="7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Q84" s="7" t="n">
-        <v>0</v>
+        <v>18964</v>
       </c>
       <c r="R84" s="7" t="n">
         <v>0</v>
@@ -6189,23 +6189,23 @@
         <v>0</v>
       </c>
       <c r="T84" s="5" t="n">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="U84" s="5" t="n">
-        <v>8625</v>
+        <v>91652</v>
       </c>
     </row>
     <row r="85" ht="18" customHeight="1">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>qrs_ekg</t>
+          <t>pr_ekg</t>
         </is>
       </c>
       <c r="B85" s="7" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="C85" s="7" t="n">
-        <v>274284</v>
+        <v>59015</v>
       </c>
       <c r="D85" s="7" t="n">
         <v>0</v>
@@ -6214,10 +6214,10 @@
         <v>0</v>
       </c>
       <c r="F85" s="7" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="G85" s="7" t="n">
-        <v>43430</v>
+        <v>0</v>
       </c>
       <c r="H85" s="7" t="n">
         <v>0</v>
@@ -6226,28 +6226,28 @@
         <v>0</v>
       </c>
       <c r="J85" s="7" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="K85" s="7" t="n">
-        <v>202581</v>
+        <v>0</v>
       </c>
       <c r="L85" s="7" t="n">
         <v>2</v>
       </c>
       <c r="M85" s="7" t="n">
-        <v>23558</v>
+        <v>23526</v>
       </c>
       <c r="N85" s="7" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="O85" s="7" t="n">
-        <v>65524</v>
+        <v>78673</v>
       </c>
       <c r="P85" s="7" t="n">
         <v>8</v>
       </c>
       <c r="Q85" s="7" t="n">
-        <v>22514</v>
+        <v>22435</v>
       </c>
       <c r="R85" s="7" t="n">
         <v>3</v>
@@ -6256,23 +6256,23 @@
         <v>500439</v>
       </c>
       <c r="T85" s="5" t="n">
-        <v>139</v>
+        <v>42</v>
       </c>
       <c r="U85" s="5" t="n">
-        <v>1132330</v>
+        <v>684088</v>
       </c>
     </row>
     <row r="86" ht="18" customHeight="1">
       <c r="A86" s="6" t="inlineStr">
         <is>
-          <t>qt_ekg</t>
+          <t>pr_qrs_qt</t>
         </is>
       </c>
       <c r="B86" s="7" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="C86" s="7" t="n">
-        <v>61199</v>
+        <v>0</v>
       </c>
       <c r="D86" s="7" t="n">
         <v>0</v>
@@ -6293,59 +6293,59 @@
         <v>0</v>
       </c>
       <c r="J86" s="7" t="n">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="K86" s="7" t="n">
-        <v>90128</v>
+        <v>66296</v>
       </c>
       <c r="L86" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M86" s="7" t="n">
-        <v>35283</v>
+        <v>0</v>
       </c>
       <c r="N86" s="7" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="O86" s="7" t="n">
-        <v>46378</v>
+        <v>0</v>
       </c>
       <c r="P86" s="7" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="Q86" s="7" t="n">
-        <v>22514</v>
+        <v>0</v>
       </c>
       <c r="R86" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S86" s="7" t="n">
-        <v>500439</v>
+        <v>0</v>
       </c>
       <c r="T86" s="5" t="n">
-        <v>54</v>
+        <v>7</v>
       </c>
       <c r="U86" s="5" t="n">
-        <v>755941</v>
+        <v>66296</v>
       </c>
     </row>
     <row r="87" ht="18" customHeight="1">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>rdbld_ct</t>
+          <t>pselectin</t>
         </is>
       </c>
       <c r="B87" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C87" s="7" t="n">
-        <v>14728</v>
+        <v>0</v>
       </c>
       <c r="D87" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E87" s="7" t="n">
-        <v>3583</v>
+        <v>326</v>
       </c>
       <c r="F87" s="7" t="n">
         <v>0</v>
@@ -6354,34 +6354,34 @@
         <v>0</v>
       </c>
       <c r="H87" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I87" s="7" t="n">
-        <v>53674</v>
+        <v>0</v>
       </c>
       <c r="J87" s="7" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="K87" s="7" t="n">
-        <v>59154</v>
+        <v>0</v>
       </c>
       <c r="L87" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M87" s="7" t="n">
-        <v>23567</v>
+        <v>0</v>
       </c>
       <c r="N87" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O87" s="7" t="n">
-        <v>3377</v>
+        <v>8299</v>
       </c>
       <c r="P87" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q87" s="7" t="n">
-        <v>3656</v>
+        <v>0</v>
       </c>
       <c r="R87" s="7" t="n">
         <v>0</v>
@@ -6390,23 +6390,23 @@
         <v>0</v>
       </c>
       <c r="T87" s="5" t="n">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="U87" s="5" t="n">
-        <v>161739</v>
+        <v>8625</v>
       </c>
     </row>
     <row r="88" ht="18" customHeight="1">
       <c r="A88" s="6" t="inlineStr">
         <is>
-          <t>rdw</t>
+          <t>qrs_ekg</t>
         </is>
       </c>
       <c r="B88" s="7" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="C88" s="7" t="n">
-        <v>12016</v>
+        <v>274284</v>
       </c>
       <c r="D88" s="7" t="n">
         <v>0</v>
@@ -6415,10 +6415,10 @@
         <v>0</v>
       </c>
       <c r="F88" s="7" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G88" s="7" t="n">
-        <v>0</v>
+        <v>43430</v>
       </c>
       <c r="H88" s="7" t="n">
         <v>0</v>
@@ -6427,65 +6427,65 @@
         <v>0</v>
       </c>
       <c r="J88" s="7" t="n">
-        <v>5</v>
+        <v>75</v>
       </c>
       <c r="K88" s="7" t="n">
-        <v>32543</v>
+        <v>202581</v>
       </c>
       <c r="L88" s="7" t="n">
         <v>2</v>
       </c>
       <c r="M88" s="7" t="n">
-        <v>23566</v>
+        <v>23558</v>
       </c>
       <c r="N88" s="7" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="O88" s="7" t="n">
-        <v>0</v>
+        <v>65524</v>
       </c>
       <c r="P88" s="7" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="Q88" s="7" t="n">
-        <v>0</v>
+        <v>22514</v>
       </c>
       <c r="R88" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S88" s="7" t="n">
-        <v>0</v>
+        <v>500439</v>
       </c>
       <c r="T88" s="5" t="n">
-        <v>11</v>
+        <v>139</v>
       </c>
       <c r="U88" s="5" t="n">
-        <v>68125</v>
+        <v>1132330</v>
       </c>
     </row>
     <row r="89" ht="18" customHeight="1">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>sleep_duration_daily</t>
+          <t>qt_ekg</t>
         </is>
       </c>
       <c r="B89" s="7" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C89" s="7" t="n">
-        <v>5925</v>
+        <v>61199</v>
       </c>
       <c r="D89" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E89" s="7" t="n">
-        <v>3529</v>
+        <v>0</v>
       </c>
       <c r="F89" s="7" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G89" s="7" t="n">
-        <v>13853</v>
+        <v>0</v>
       </c>
       <c r="H89" s="7" t="n">
         <v>0</v>
@@ -6494,59 +6494,59 @@
         <v>0</v>
       </c>
       <c r="J89" s="7" t="n">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="K89" s="7" t="n">
-        <v>129670</v>
+        <v>90128</v>
       </c>
       <c r="L89" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M89" s="7" t="n">
-        <v>23080</v>
+        <v>35283</v>
       </c>
       <c r="N89" s="7" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="O89" s="7" t="n">
-        <v>6955</v>
+        <v>46378</v>
       </c>
       <c r="P89" s="7" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="Q89" s="7" t="n">
-        <v>10941</v>
+        <v>22514</v>
       </c>
       <c r="R89" s="7" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="S89" s="7" t="n">
-        <v>626832</v>
+        <v>500439</v>
       </c>
       <c r="T89" s="5" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="U89" s="5" t="n">
-        <v>820785</v>
+        <v>755941</v>
       </c>
     </row>
     <row r="90" ht="18" customHeight="1">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>sodium_blood</t>
+          <t>rdbld_ct</t>
         </is>
       </c>
       <c r="B90" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C90" s="7" t="n">
-        <v>52984</v>
+        <v>14728</v>
       </c>
       <c r="D90" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E90" s="7" t="n">
-        <v>0</v>
+        <v>3583</v>
       </c>
       <c r="F90" s="7" t="n">
         <v>0</v>
@@ -6555,89 +6555,89 @@
         <v>0</v>
       </c>
       <c r="H90" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I90" s="7" t="n">
-        <v>0</v>
+        <v>53674</v>
       </c>
       <c r="J90" s="7" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="K90" s="7" t="n">
-        <v>17171</v>
+        <v>59154</v>
       </c>
       <c r="L90" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M90" s="7" t="n">
-        <v>0</v>
+        <v>23567</v>
       </c>
       <c r="N90" s="7" t="n">
         <v>1</v>
       </c>
       <c r="O90" s="7" t="n">
-        <v>3839</v>
+        <v>3377</v>
       </c>
       <c r="P90" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q90" s="7" t="n">
-        <v>6129</v>
+        <v>3656</v>
       </c>
       <c r="R90" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S90" s="7" t="n">
-        <v>5721</v>
+        <v>0</v>
       </c>
       <c r="T90" s="5" t="n">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="U90" s="5" t="n">
-        <v>85844</v>
+        <v>161739</v>
       </c>
     </row>
     <row r="91" ht="18" customHeight="1">
       <c r="A91" s="6" t="inlineStr">
         <is>
-          <t>sodium_intak</t>
+          <t>rdw</t>
         </is>
       </c>
       <c r="B91" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C91" s="7" t="n">
-        <v>28614</v>
+        <v>12016</v>
       </c>
       <c r="D91" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E91" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F91" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G91" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H91" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I91" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J91" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="E91" s="7" t="n">
-        <v>16962</v>
-      </c>
-      <c r="F91" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="G91" s="7" t="n">
-        <v>12180</v>
-      </c>
-      <c r="H91" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I91" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J91" s="7" t="n">
-        <v>18</v>
-      </c>
       <c r="K91" s="7" t="n">
-        <v>82860</v>
+        <v>32543</v>
       </c>
       <c r="L91" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M91" s="7" t="n">
-        <v>0</v>
+        <v>23566</v>
       </c>
       <c r="N91" s="7" t="n">
         <v>0</v>
@@ -6646,102 +6646,102 @@
         <v>0</v>
       </c>
       <c r="P91" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q91" s="7" t="n">
-        <v>4252</v>
+        <v>0</v>
       </c>
       <c r="R91" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S91" s="7" t="n">
-        <v>338044</v>
+        <v>0</v>
       </c>
       <c r="T91" s="5" t="n">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="U91" s="5" t="n">
-        <v>482912</v>
+        <v>68125</v>
       </c>
     </row>
     <row r="92" ht="18" customHeight="1">
       <c r="A92" s="6" t="inlineStr">
         <is>
-          <t>spirometry</t>
+          <t>sleep_duration_daily</t>
         </is>
       </c>
       <c r="B92" s="7" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="C92" s="7" t="n">
-        <v>226242</v>
+        <v>5925</v>
       </c>
       <c r="D92" s="7" t="n">
-        <v>47</v>
+        <v>2</v>
       </c>
       <c r="E92" s="7" t="n">
-        <v>118442</v>
+        <v>3529</v>
       </c>
       <c r="F92" s="7" t="n">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="G92" s="7" t="n">
-        <v>77987</v>
+        <v>13853</v>
       </c>
       <c r="H92" s="7" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="I92" s="7" t="n">
-        <v>264146</v>
+        <v>0</v>
       </c>
       <c r="J92" s="7" t="n">
-        <v>63</v>
+        <v>31</v>
       </c>
       <c r="K92" s="7" t="n">
-        <v>186708</v>
+        <v>129670</v>
       </c>
       <c r="L92" s="7" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="M92" s="7" t="n">
-        <v>79778</v>
+        <v>23080</v>
       </c>
       <c r="N92" s="7" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="O92" s="7" t="n">
-        <v>44329</v>
+        <v>6955</v>
       </c>
       <c r="P92" s="7" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="Q92" s="7" t="n">
-        <v>28584</v>
+        <v>10941</v>
       </c>
       <c r="R92" s="7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S92" s="7" t="n">
-        <v>0</v>
+        <v>626832</v>
       </c>
       <c r="T92" s="5" t="n">
-        <v>211</v>
+        <v>55</v>
       </c>
       <c r="U92" s="5" t="n">
-        <v>1026216</v>
+        <v>820785</v>
       </c>
     </row>
     <row r="93" ht="18" customHeight="1">
       <c r="A93" s="6" t="inlineStr">
         <is>
-          <t>spo2</t>
+          <t>sodium_blood</t>
         </is>
       </c>
       <c r="B93" s="7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C93" s="7" t="n">
-        <v>0</v>
+        <v>52984</v>
       </c>
       <c r="D93" s="7" t="n">
         <v>0</v>
@@ -6750,77 +6750,77 @@
         <v>0</v>
       </c>
       <c r="F93" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G93" s="7" t="n">
-        <v>10480</v>
+        <v>0</v>
       </c>
       <c r="H93" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I93" s="7" t="n">
-        <v>64224</v>
+        <v>0</v>
       </c>
       <c r="J93" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="K93" s="7" t="n">
+        <v>17171</v>
+      </c>
+      <c r="L93" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M93" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N93" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="K93" s="7" t="n">
-        <v>715</v>
-      </c>
-      <c r="L93" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="M93" s="7" t="n">
-        <v>22347</v>
-      </c>
-      <c r="N93" s="7" t="n">
-        <v>0</v>
-      </c>
       <c r="O93" s="7" t="n">
-        <v>0</v>
+        <v>3839</v>
       </c>
       <c r="P93" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q93" s="7" t="n">
-        <v>0</v>
+        <v>6129</v>
       </c>
       <c r="R93" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S93" s="7" t="n">
-        <v>0</v>
+        <v>5721</v>
       </c>
       <c r="T93" s="5" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="U93" s="5" t="n">
-        <v>97766</v>
+        <v>85844</v>
       </c>
     </row>
     <row r="94" ht="18" customHeight="1">
       <c r="A94" s="6" t="inlineStr">
         <is>
-          <t>tnfa</t>
+          <t>sodium_intak</t>
         </is>
       </c>
       <c r="B94" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C94" s="7" t="n">
-        <v>0</v>
+        <v>28614</v>
       </c>
       <c r="D94" s="7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E94" s="7" t="n">
-        <v>0</v>
+        <v>16962</v>
       </c>
       <c r="F94" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G94" s="7" t="n">
-        <v>0</v>
+        <v>12180</v>
       </c>
       <c r="H94" s="7" t="n">
         <v>0</v>
@@ -6829,10 +6829,10 @@
         <v>0</v>
       </c>
       <c r="J94" s="7" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="K94" s="7" t="n">
-        <v>0</v>
+        <v>82860</v>
       </c>
       <c r="L94" s="7" t="n">
         <v>0</v>
@@ -6847,28 +6847,28 @@
         <v>0</v>
       </c>
       <c r="P94" s="7" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q94" s="7" t="n">
-        <v>6524</v>
+        <v>4252</v>
       </c>
       <c r="R94" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S94" s="7" t="n">
-        <v>0</v>
+        <v>338044</v>
       </c>
       <c r="T94" s="5" t="n">
-        <v>6</v>
+        <v>31</v>
       </c>
       <c r="U94" s="5" t="n">
-        <v>6524</v>
+        <v>482912</v>
       </c>
     </row>
     <row r="95" ht="18" customHeight="1">
       <c r="A95" s="6" t="inlineStr">
         <is>
-          <t>tnfa_r1</t>
+          <t>spo2</t>
         </is>
       </c>
       <c r="B95" s="7" t="n">
@@ -6884,28 +6884,28 @@
         <v>0</v>
       </c>
       <c r="F95" s="7" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G95" s="7" t="n">
-        <v>0</v>
+        <v>10480</v>
       </c>
       <c r="H95" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I95" s="7" t="n">
-        <v>0</v>
+        <v>64224</v>
       </c>
       <c r="J95" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K95" s="7" t="n">
-        <v>0</v>
+        <v>715</v>
       </c>
       <c r="L95" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M95" s="7" t="n">
-        <v>0</v>
+        <v>22347</v>
       </c>
       <c r="N95" s="7" t="n">
         <v>0</v>
@@ -6914,10 +6914,10 @@
         <v>0</v>
       </c>
       <c r="P95" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q95" s="7" t="n">
-        <v>9242</v>
+        <v>0</v>
       </c>
       <c r="R95" s="7" t="n">
         <v>0</v>
@@ -6926,35 +6926,35 @@
         <v>0</v>
       </c>
       <c r="T95" s="5" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="U95" s="5" t="n">
-        <v>9242</v>
+        <v>97766</v>
       </c>
     </row>
     <row r="96" ht="18" customHeight="1">
       <c r="A96" s="6" t="inlineStr">
         <is>
-          <t>tot_chol_bld</t>
+          <t>tnfa</t>
         </is>
       </c>
       <c r="B96" s="7" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="C96" s="7" t="n">
-        <v>245458</v>
+        <v>0</v>
       </c>
       <c r="D96" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E96" s="7" t="n">
-        <v>6897</v>
+        <v>0</v>
       </c>
       <c r="F96" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G96" s="7" t="n">
-        <v>11010</v>
+        <v>0</v>
       </c>
       <c r="H96" s="7" t="n">
         <v>0</v>
@@ -6963,65 +6963,65 @@
         <v>0</v>
       </c>
       <c r="J96" s="7" t="n">
-        <v>64</v>
+        <v>0</v>
       </c>
       <c r="K96" s="7" t="n">
-        <v>218271</v>
+        <v>0</v>
       </c>
       <c r="L96" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M96" s="7" t="n">
-        <v>23653</v>
+        <v>0</v>
       </c>
       <c r="N96" s="7" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="O96" s="7" t="n">
-        <v>31460</v>
+        <v>0</v>
       </c>
       <c r="P96" s="7" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="Q96" s="7" t="n">
-        <v>68149</v>
+        <v>6524</v>
       </c>
       <c r="R96" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S96" s="7" t="n">
-        <v>46610</v>
+        <v>0</v>
       </c>
       <c r="T96" s="5" t="n">
-        <v>131</v>
+        <v>6</v>
       </c>
       <c r="U96" s="5" t="n">
-        <v>651508</v>
+        <v>6524</v>
       </c>
     </row>
     <row r="97" ht="18" customHeight="1">
       <c r="A97" s="6" t="inlineStr">
         <is>
-          <t>triglyc_bld</t>
+          <t>tnfa_r1</t>
         </is>
       </c>
       <c r="B97" s="7" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="C97" s="7" t="n">
-        <v>167017</v>
+        <v>0</v>
       </c>
       <c r="D97" s="7" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E97" s="7" t="n">
-        <v>16569</v>
+        <v>0</v>
       </c>
       <c r="F97" s="7" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G97" s="7" t="n">
-        <v>29264</v>
+        <v>0</v>
       </c>
       <c r="H97" s="7" t="n">
         <v>0</v>
@@ -7030,65 +7030,65 @@
         <v>0</v>
       </c>
       <c r="J97" s="7" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="K97" s="7" t="n">
-        <v>168009</v>
+        <v>0</v>
       </c>
       <c r="L97" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M97" s="7" t="n">
-        <v>23653</v>
+        <v>0</v>
       </c>
       <c r="N97" s="7" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="O97" s="7" t="n">
-        <v>32777</v>
+        <v>0</v>
       </c>
       <c r="P97" s="7" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="Q97" s="7" t="n">
-        <v>67803</v>
+        <v>9242</v>
       </c>
       <c r="R97" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S97" s="7" t="n">
-        <v>46610</v>
+        <v>0</v>
       </c>
       <c r="T97" s="5" t="n">
-        <v>117</v>
+        <v>2</v>
       </c>
       <c r="U97" s="5" t="n">
-        <v>551702</v>
+        <v>9242</v>
       </c>
     </row>
     <row r="98" ht="18" customHeight="1">
       <c r="A98" s="6" t="inlineStr">
         <is>
-          <t>troponin</t>
+          <t>tot_chol_bld</t>
         </is>
       </c>
       <c r="B98" s="7" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="C98" s="7" t="n">
-        <v>59241</v>
+        <v>245458</v>
       </c>
       <c r="D98" s="7" t="n">
         <v>2</v>
       </c>
       <c r="E98" s="7" t="n">
-        <v>77</v>
+        <v>6897</v>
       </c>
       <c r="F98" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G98" s="7" t="n">
-        <v>0</v>
+        <v>11010</v>
       </c>
       <c r="H98" s="7" t="n">
         <v>0</v>
@@ -7097,65 +7097,65 @@
         <v>0</v>
       </c>
       <c r="J98" s="7" t="n">
-        <v>4</v>
+        <v>64</v>
       </c>
       <c r="K98" s="7" t="n">
-        <v>14391</v>
+        <v>218271</v>
       </c>
       <c r="L98" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M98" s="7" t="n">
-        <v>0</v>
+        <v>23653</v>
       </c>
       <c r="N98" s="7" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="O98" s="7" t="n">
-        <v>0</v>
+        <v>31460</v>
       </c>
       <c r="P98" s="7" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="Q98" s="7" t="n">
-        <v>0</v>
+        <v>68149</v>
       </c>
       <c r="R98" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="S98" s="7" t="n">
-        <v>4604</v>
+        <v>46610</v>
       </c>
       <c r="T98" s="5" t="n">
-        <v>18</v>
+        <v>131</v>
       </c>
       <c r="U98" s="5" t="n">
-        <v>78313</v>
+        <v>651508</v>
       </c>
     </row>
     <row r="99" ht="18" customHeight="1">
       <c r="A99" s="6" t="inlineStr">
         <is>
-          <t>vege_serving</t>
+          <t>triglyc_bld</t>
         </is>
       </c>
       <c r="B99" s="7" t="n">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="C99" s="7" t="n">
-        <v>322380</v>
+        <v>167017</v>
       </c>
       <c r="D99" s="7" t="n">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="E99" s="7" t="n">
-        <v>74514</v>
+        <v>16569</v>
       </c>
       <c r="F99" s="7" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G99" s="7" t="n">
-        <v>771</v>
+        <v>29264</v>
       </c>
       <c r="H99" s="7" t="n">
         <v>0</v>
@@ -7164,132 +7164,132 @@
         <v>0</v>
       </c>
       <c r="J99" s="7" t="n">
-        <v>232</v>
+        <v>50</v>
       </c>
       <c r="K99" s="7" t="n">
-        <v>638568</v>
+        <v>168009</v>
       </c>
       <c r="L99" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M99" s="7" t="n">
-        <v>0</v>
+        <v>23653</v>
       </c>
       <c r="N99" s="7" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="O99" s="7" t="n">
-        <v>7594</v>
+        <v>32777</v>
       </c>
       <c r="P99" s="7" t="n">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="Q99" s="7" t="n">
-        <v>29869</v>
+        <v>67803</v>
       </c>
       <c r="R99" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S99" s="7" t="n">
-        <v>680137</v>
+        <v>46610</v>
       </c>
       <c r="T99" s="5" t="n">
-        <v>300</v>
+        <v>117</v>
       </c>
       <c r="U99" s="5" t="n">
-        <v>1753833</v>
+        <v>551702</v>
       </c>
     </row>
     <row r="100" ht="18" customHeight="1">
       <c r="A100" s="6" t="inlineStr">
         <is>
-          <t>waist_circ</t>
+          <t>troponin</t>
         </is>
       </c>
       <c r="B100" s="7" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="C100" s="7" t="n">
-        <v>54019</v>
+        <v>59241</v>
       </c>
       <c r="D100" s="7" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="E100" s="7" t="n">
-        <v>30185</v>
+        <v>77</v>
       </c>
       <c r="F100" s="7" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="G100" s="7" t="n">
-        <v>43939</v>
+        <v>0</v>
       </c>
       <c r="H100" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I100" s="7" t="n">
-        <v>53850</v>
+        <v>0</v>
       </c>
       <c r="J100" s="7" t="n">
-        <v>55</v>
+        <v>4</v>
       </c>
       <c r="K100" s="7" t="n">
-        <v>175209</v>
+        <v>14391</v>
       </c>
       <c r="L100" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M100" s="7" t="n">
-        <v>23633</v>
+        <v>0</v>
       </c>
       <c r="N100" s="7" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="O100" s="7" t="n">
-        <v>25409</v>
+        <v>0</v>
       </c>
       <c r="P100" s="7" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="Q100" s="7" t="n">
-        <v>56543</v>
+        <v>0</v>
       </c>
       <c r="R100" s="7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="S100" s="7" t="n">
-        <v>1619039</v>
+        <v>4604</v>
       </c>
       <c r="T100" s="5" t="n">
-        <v>112</v>
+        <v>18</v>
       </c>
       <c r="U100" s="5" t="n">
-        <v>2081826</v>
+        <v>78313</v>
       </c>
     </row>
     <row r="101" ht="18" customHeight="1">
       <c r="A101" s="6" t="inlineStr">
         <is>
-          <t>waist_hip</t>
+          <t>vege_serving</t>
         </is>
       </c>
       <c r="B101" s="7" t="n">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="C101" s="7" t="n">
-        <v>106654</v>
+        <v>322380</v>
       </c>
       <c r="D101" s="7" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="E101" s="7" t="n">
-        <v>388</v>
+        <v>74514</v>
       </c>
       <c r="F101" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G101" s="7" t="n">
-        <v>0</v>
+        <v>771</v>
       </c>
       <c r="H101" s="7" t="n">
         <v>0</v>
@@ -7298,241 +7298,375 @@
         <v>0</v>
       </c>
       <c r="J101" s="7" t="n">
-        <v>0</v>
+        <v>232</v>
       </c>
       <c r="K101" s="7" t="n">
-        <v>0</v>
+        <v>638568</v>
       </c>
       <c r="L101" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M101" s="7" t="n">
-        <v>23626</v>
+        <v>0</v>
       </c>
       <c r="N101" s="7" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="O101" s="7" t="n">
-        <v>23478</v>
+        <v>7594</v>
       </c>
       <c r="P101" s="7" t="n">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="Q101" s="7" t="n">
-        <v>89497</v>
+        <v>29869</v>
       </c>
       <c r="R101" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S101" s="7" t="n">
-        <v>1610605</v>
+        <v>680137</v>
       </c>
       <c r="T101" s="5" t="n">
-        <v>51</v>
+        <v>300</v>
       </c>
       <c r="U101" s="5" t="n">
-        <v>1854248</v>
+        <v>1753833</v>
       </c>
     </row>
     <row r="102" ht="18" customHeight="1">
       <c r="A102" s="6" t="inlineStr">
         <is>
-          <t>whtbld_ct</t>
+          <t>waist_circ</t>
         </is>
       </c>
       <c r="B102" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C102" s="7" t="n">
-        <v>43076</v>
+        <v>54019</v>
       </c>
       <c r="D102" s="7" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E102" s="7" t="n">
-        <v>3583</v>
+        <v>30185</v>
       </c>
       <c r="F102" s="7" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="G102" s="7" t="n">
-        <v>10978</v>
+        <v>43939</v>
       </c>
       <c r="H102" s="7" t="n">
         <v>3</v>
       </c>
       <c r="I102" s="7" t="n">
-        <v>53674</v>
+        <v>53850</v>
       </c>
       <c r="J102" s="7" t="n">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="K102" s="7" t="n">
-        <v>60160</v>
+        <v>175209</v>
       </c>
       <c r="L102" s="7" t="n">
         <v>2</v>
       </c>
       <c r="M102" s="7" t="n">
-        <v>22911</v>
+        <v>23633</v>
       </c>
       <c r="N102" s="7" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="O102" s="7" t="n">
-        <v>3377</v>
+        <v>25409</v>
       </c>
       <c r="P102" s="7" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="Q102" s="7" t="n">
-        <v>3656</v>
+        <v>56543</v>
       </c>
       <c r="R102" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S102" s="7" t="n">
-        <v>623680</v>
+        <v>1619039</v>
       </c>
       <c r="T102" s="5" t="n">
-        <v>32</v>
+        <v>112</v>
       </c>
       <c r="U102" s="5" t="n">
-        <v>825095</v>
+        <v>2081826</v>
       </c>
     </row>
     <row r="103" ht="18" customHeight="1">
       <c r="A103" s="6" t="inlineStr">
         <is>
+          <t>waist_hip</t>
+        </is>
+      </c>
+      <c r="B103" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="C103" s="7" t="n">
+        <v>106654</v>
+      </c>
+      <c r="D103" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E103" s="7" t="n">
+        <v>388</v>
+      </c>
+      <c r="F103" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G103" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H103" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I103" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J103" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K103" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L103" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="M103" s="7" t="n">
+        <v>23626</v>
+      </c>
+      <c r="N103" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="O103" s="7" t="n">
+        <v>23478</v>
+      </c>
+      <c r="P103" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="Q103" s="7" t="n">
+        <v>89497</v>
+      </c>
+      <c r="R103" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="S103" s="7" t="n">
+        <v>1610605</v>
+      </c>
+      <c r="T103" s="5" t="n">
+        <v>51</v>
+      </c>
+      <c r="U103" s="5" t="n">
+        <v>1854248</v>
+      </c>
+    </row>
+    <row r="104" ht="18" customHeight="1">
+      <c r="A104" s="6" t="inlineStr">
+        <is>
+          <t>whtbld_ct</t>
+        </is>
+      </c>
+      <c r="B104" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C104" s="7" t="n">
+        <v>43076</v>
+      </c>
+      <c r="D104" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E104" s="7" t="n">
+        <v>3583</v>
+      </c>
+      <c r="F104" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G104" s="7" t="n">
+        <v>10978</v>
+      </c>
+      <c r="H104" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="I104" s="7" t="n">
+        <v>53674</v>
+      </c>
+      <c r="J104" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="K104" s="7" t="n">
+        <v>60160</v>
+      </c>
+      <c r="L104" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="M104" s="7" t="n">
+        <v>22911</v>
+      </c>
+      <c r="N104" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="O104" s="7" t="n">
+        <v>3377</v>
+      </c>
+      <c r="P104" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q104" s="7" t="n">
+        <v>3656</v>
+      </c>
+      <c r="R104" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="S104" s="7" t="n">
+        <v>623680</v>
+      </c>
+      <c r="T104" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="U104" s="5" t="n">
+        <v>825095</v>
+      </c>
+    </row>
+    <row r="105" ht="18" customHeight="1">
+      <c r="A105" s="6" t="inlineStr">
+        <is>
           <t>willeb_fac</t>
         </is>
       </c>
-      <c r="B103" s="7" t="n">
+      <c r="B105" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="C103" s="7" t="n">
+      <c r="C105" s="7" t="n">
         <v>14801</v>
       </c>
-      <c r="D103" s="7" t="n">
+      <c r="D105" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="E103" s="7" t="n">
+      <c r="E105" s="7" t="n">
         <v>6928</v>
       </c>
-      <c r="F103" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G103" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H103" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I103" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J103" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="K103" s="7" t="n">
+      <c r="F105" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G105" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H105" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I105" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J105" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="K105" s="7" t="n">
         <v>12072</v>
       </c>
-      <c r="L103" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M103" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N103" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O103" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P103" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q103" s="7" t="n">
+      <c r="L105" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M105" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N105" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O105" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P105" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q105" s="7" t="n">
         <v>7391</v>
       </c>
-      <c r="R103" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="S103" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="T103" s="5" t="n">
+      <c r="R105" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S105" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T105" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="U103" s="5" t="n">
+      <c r="U105" s="5" t="n">
         <v>41192</v>
       </c>
     </row>
-    <row r="104" ht="18" customHeight="1">
-      <c r="A104" s="8" t="inlineStr">
+    <row r="106" ht="18" customHeight="1">
+      <c r="A106" s="8" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B104" s="9" t="n">
-        <v>1178</v>
-      </c>
-      <c r="C104" s="9" t="n">
-        <v>11553653</v>
-      </c>
-      <c r="D104" s="9" t="n">
-        <v>565</v>
-      </c>
-      <c r="E104" s="9" t="n">
-        <v>1035671</v>
-      </c>
-      <c r="F104" s="9" t="n">
-        <v>1349</v>
-      </c>
-      <c r="G104" s="9" t="n">
-        <v>4161858</v>
-      </c>
-      <c r="H104" s="9" t="n">
-        <v>112</v>
-      </c>
-      <c r="I104" s="9" t="n">
-        <v>2122662</v>
-      </c>
-      <c r="J104" s="9" t="n">
-        <v>3087</v>
-      </c>
-      <c r="K104" s="9" t="n">
-        <v>9071383</v>
-      </c>
-      <c r="L104" s="9" t="n">
-        <v>165</v>
-      </c>
-      <c r="M104" s="9" t="n">
-        <v>1772032</v>
-      </c>
-      <c r="N104" s="9" t="n">
-        <v>477</v>
-      </c>
-      <c r="O104" s="9" t="n">
-        <v>1643015</v>
-      </c>
-      <c r="P104" s="9" t="n">
-        <v>1196</v>
-      </c>
-      <c r="Q104" s="9" t="n">
-        <v>3908574</v>
-      </c>
-      <c r="R104" s="9" t="n">
+      <c r="B106" s="9" t="n">
+        <v>1180</v>
+      </c>
+      <c r="C106" s="9" t="n">
+        <v>11570834</v>
+      </c>
+      <c r="D106" s="9" t="n">
+        <v>566</v>
+      </c>
+      <c r="E106" s="9" t="n">
+        <v>1038752</v>
+      </c>
+      <c r="F106" s="9" t="n">
+        <v>1346</v>
+      </c>
+      <c r="G106" s="9" t="n">
+        <v>4149685</v>
+      </c>
+      <c r="H106" s="9" t="n">
+        <v>111</v>
+      </c>
+      <c r="I106" s="9" t="n">
+        <v>2104709</v>
+      </c>
+      <c r="J106" s="9" t="n">
+        <v>3109</v>
+      </c>
+      <c r="K106" s="9" t="n">
+        <v>9247109</v>
+      </c>
+      <c r="L106" s="9" t="n">
+        <v>167</v>
+      </c>
+      <c r="M106" s="9" t="n">
+        <v>1795694</v>
+      </c>
+      <c r="N106" s="9" t="n">
+        <v>476</v>
+      </c>
+      <c r="O106" s="9" t="n">
+        <v>1639132</v>
+      </c>
+      <c r="P106" s="9" t="n">
+        <v>1201</v>
+      </c>
+      <c r="Q106" s="9" t="n">
+        <v>3916957</v>
+      </c>
+      <c r="R106" s="9" t="n">
         <v>360</v>
       </c>
-      <c r="S104" s="9" t="n">
+      <c r="S106" s="9" t="n">
         <v>34121402</v>
       </c>
-      <c r="T104" s="9" t="n">
-        <v>8489</v>
-      </c>
-      <c r="U104" s="9" t="n">
-        <v>69390250</v>
+      <c r="T106" s="9" t="n">
+        <v>8516</v>
+      </c>
+      <c r="U106" s="9" t="n">
+        <v>69584274</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix OMOP code mapping for spirometry concepts
Correct SPIROMETRY_OMOP_MAP to use only one code per concept:
FEV1 → OMOP:4241837, FVC → OMOP:4176265, FEV1/FVC → OMOP:3011505

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tables/before_table.xlsx
+++ b/tables/before_table.xlsx
@@ -3589,52 +3589,52 @@
         </is>
       </c>
       <c r="B46" s="7" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C46" s="7" t="n">
-        <v>87503</v>
+        <v>52873</v>
       </c>
       <c r="D46" s="7" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E46" s="7" t="n">
-        <v>64098</v>
+        <v>57425</v>
       </c>
       <c r="F46" s="7" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G46" s="7" t="n">
-        <v>31282</v>
+        <v>20005</v>
       </c>
       <c r="H46" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I46" s="7" t="n">
-        <v>82063</v>
+        <v>61881</v>
       </c>
       <c r="J46" s="7" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="K46" s="7" t="n">
-        <v>124086</v>
+        <v>127166</v>
       </c>
       <c r="L46" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M46" s="7" t="n">
-        <v>34509</v>
+        <v>23178</v>
       </c>
       <c r="N46" s="7" t="n">
         <v>4</v>
       </c>
       <c r="O46" s="7" t="n">
-        <v>14702</v>
+        <v>14700</v>
       </c>
       <c r="P46" s="7" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="Q46" s="7" t="n">
-        <v>12201</v>
+        <v>8427</v>
       </c>
       <c r="R46" s="7" t="n">
         <v>0</v>
@@ -3643,10 +3643,10 @@
         <v>0</v>
       </c>
       <c r="T46" s="5" t="n">
-        <v>94</v>
+        <v>81</v>
       </c>
       <c r="U46" s="5" t="n">
-        <v>450444</v>
+        <v>365655</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
@@ -3656,10 +3656,10 @@
         </is>
       </c>
       <c r="B47" s="7" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C47" s="7" t="n">
-        <v>82611</v>
+        <v>43161</v>
       </c>
       <c r="D47" s="7" t="n">
         <v>0</v>
@@ -3668,16 +3668,16 @@
         <v>0</v>
       </c>
       <c r="F47" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G47" s="7" t="n">
-        <v>9673</v>
+        <v>4819</v>
       </c>
       <c r="H47" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I47" s="7" t="n">
-        <v>82063</v>
+        <v>61877</v>
       </c>
       <c r="J47" s="7" t="n">
         <v>24</v>
@@ -3686,10 +3686,10 @@
         <v>111182</v>
       </c>
       <c r="L47" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M47" s="7" t="n">
-        <v>34422</v>
+        <v>23077</v>
       </c>
       <c r="N47" s="7" t="n">
         <v>3</v>
@@ -3698,10 +3698,10 @@
         <v>11044</v>
       </c>
       <c r="P47" s="7" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="Q47" s="7" t="n">
-        <v>12550</v>
+        <v>8410</v>
       </c>
       <c r="R47" s="7" t="n">
         <v>0</v>
@@ -3710,10 +3710,10 @@
         <v>0</v>
       </c>
       <c r="T47" s="5" t="n">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="U47" s="5" t="n">
-        <v>343545</v>
+        <v>263570</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
@@ -3857,52 +3857,52 @@
         </is>
       </c>
       <c r="B50" s="7" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C50" s="7" t="n">
-        <v>73309</v>
+        <v>52873</v>
       </c>
       <c r="D50" s="7" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E50" s="7" t="n">
-        <v>57425</v>
+        <v>64098</v>
       </c>
       <c r="F50" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G50" s="7" t="n">
-        <v>24859</v>
+        <v>20004</v>
       </c>
       <c r="H50" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I50" s="7" t="n">
-        <v>82067</v>
+        <v>61877</v>
       </c>
       <c r="J50" s="7" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="K50" s="7" t="n">
-        <v>127166</v>
+        <v>124086</v>
       </c>
       <c r="L50" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M50" s="7" t="n">
-        <v>34509</v>
+        <v>23178</v>
       </c>
       <c r="N50" s="7" t="n">
         <v>4</v>
       </c>
       <c r="O50" s="7" t="n">
-        <v>14700</v>
+        <v>14702</v>
       </c>
       <c r="P50" s="7" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="Q50" s="7" t="n">
-        <v>12216</v>
+        <v>8412</v>
       </c>
       <c r="R50" s="7" t="n">
         <v>0</v>
@@ -3911,10 +3911,10 @@
         <v>0</v>
       </c>
       <c r="T50" s="5" t="n">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="U50" s="5" t="n">
-        <v>426251</v>
+        <v>369230</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
@@ -7609,10 +7609,10 @@
         </is>
       </c>
       <c r="B106" s="9" t="n">
-        <v>1180</v>
+        <v>1167</v>
       </c>
       <c r="C106" s="9" t="n">
-        <v>11570834</v>
+        <v>11476318</v>
       </c>
       <c r="D106" s="9" t="n">
         <v>566</v>
@@ -7621,16 +7621,16 @@
         <v>1038752</v>
       </c>
       <c r="F106" s="9" t="n">
-        <v>1346</v>
+        <v>1341</v>
       </c>
       <c r="G106" s="9" t="n">
-        <v>4149685</v>
+        <v>4128699</v>
       </c>
       <c r="H106" s="9" t="n">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="I106" s="9" t="n">
-        <v>2104709</v>
+        <v>2044151</v>
       </c>
       <c r="J106" s="9" t="n">
         <v>3109</v>
@@ -7639,10 +7639,10 @@
         <v>9247109</v>
       </c>
       <c r="L106" s="9" t="n">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="M106" s="9" t="n">
-        <v>1795694</v>
+        <v>1761687</v>
       </c>
       <c r="N106" s="9" t="n">
         <v>476</v>
@@ -7651,10 +7651,10 @@
         <v>1639132</v>
       </c>
       <c r="P106" s="9" t="n">
-        <v>1201</v>
+        <v>1192</v>
       </c>
       <c r="Q106" s="9" t="n">
-        <v>3916957</v>
+        <v>3905239</v>
       </c>
       <c r="R106" s="9" t="n">
         <v>360</v>
@@ -7663,10 +7663,10 @@
         <v>34121402</v>
       </c>
       <c r="T106" s="9" t="n">
-        <v>8516</v>
+        <v>8483</v>
       </c>
       <c r="U106" s="9" t="n">
-        <v>69584274</v>
+        <v>69362489</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Exclude chr_bronchitis, emphysema, hypert_trt, hist_cor_bypg from Conditions row
These files remain in Drug Exposures/Procedures for cohorts that classify them there.
Conditions total: 2,075 → 1,990 vars; 17,889,081 → 17,186,916 data pts.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tables/before_table.xlsx
+++ b/tables/before_table.xlsx
@@ -647,10 +647,10 @@
         <v>4868066</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>191561</v>
+        <v>154410</v>
       </c>
       <c r="F2" s="4" t="n">
         <v>287</v>
@@ -659,22 +659,22 @@
         <v>878051</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>357328</v>
+        <v>331148</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>662</v>
+        <v>611</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>1580952</v>
+        <v>1496855</v>
       </c>
       <c r="L2" s="4" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="M2" s="4" t="n">
-        <v>278943</v>
+        <v>267228</v>
       </c>
       <c r="N2" s="4" t="n">
         <v>107</v>
@@ -683,22 +683,22 @@
         <v>474003</v>
       </c>
       <c r="P2" s="4" t="n">
-        <v>152</v>
+        <v>143</v>
       </c>
       <c r="Q2" s="4" t="n">
-        <v>680731</v>
+        <v>648521</v>
       </c>
       <c r="R2" s="4" t="n">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="S2" s="4" t="n">
-        <v>8579446</v>
+        <v>8068634</v>
       </c>
       <c r="T2" s="5" t="n">
-        <v>2075</v>
+        <v>1990</v>
       </c>
       <c r="U2" s="5" t="n">
-        <v>17889081</v>
+        <v>17186916</v>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
@@ -7548,10 +7548,10 @@
         <v>11476318</v>
       </c>
       <c r="D105" s="9" t="n">
-        <v>566</v>
+        <v>551</v>
       </c>
       <c r="E105" s="9" t="n">
-        <v>1038752</v>
+        <v>1001601</v>
       </c>
       <c r="F105" s="9" t="n">
         <v>1341</v>
@@ -7560,22 +7560,22 @@
         <v>4128699</v>
       </c>
       <c r="H105" s="9" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="I105" s="9" t="n">
-        <v>2088195</v>
+        <v>2062015</v>
       </c>
       <c r="J105" s="9" t="n">
-        <v>3109</v>
+        <v>3058</v>
       </c>
       <c r="K105" s="9" t="n">
-        <v>9247109</v>
+        <v>9163012</v>
       </c>
       <c r="L105" s="9" t="n">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="M105" s="9" t="n">
-        <v>1761687</v>
+        <v>1749972</v>
       </c>
       <c r="N105" s="9" t="n">
         <v>476</v>
@@ -7584,22 +7584,22 @@
         <v>1639132</v>
       </c>
       <c r="P105" s="9" t="n">
-        <v>1192</v>
+        <v>1183</v>
       </c>
       <c r="Q105" s="9" t="n">
-        <v>3905239</v>
+        <v>3873029</v>
       </c>
       <c r="R105" s="9" t="n">
-        <v>360</v>
+        <v>353</v>
       </c>
       <c r="S105" s="9" t="n">
-        <v>34121402</v>
+        <v>33610590</v>
       </c>
       <c r="T105" s="9" t="n">
-        <v>8485</v>
+        <v>8400</v>
       </c>
       <c r="U105" s="9" t="n">
-        <v>69406533</v>
+        <v>68704368</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Force pacem_stat into Procedures row for all cohorts
ARIC/HCHS/MESA use MeasurementObservation for pacem_stat; override to Procedures
to match WHI. ARIC Procedures: 17 → 20 vars. Table: 103 rows (99 continuous).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tables/before_table.xlsx
+++ b/tables/before_table.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U105"/>
+  <dimension ref="A1:U104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -775,10 +775,10 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>113048</v>
+        <v>126158</v>
       </c>
       <c r="D4" s="4" t="n">
         <v>2</v>
@@ -805,10 +805,10 @@
         <v>28154</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>0</v>
+        <v>11848</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>14</v>
@@ -817,10 +817,10 @@
         <v>11088</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>0</v>
+        <v>12922</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>13</v>
@@ -829,10 +829,10 @@
         <v>1236045</v>
       </c>
       <c r="T4" s="5" t="n">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="U4" s="5" t="n">
-        <v>1487492</v>
+        <v>1525372</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
@@ -5863,160 +5863,160 @@
     <row r="80" ht="18" customHeight="1">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>pacem_stat</t>
+          <t>platelet_ct</t>
         </is>
       </c>
       <c r="B80" s="7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C80" s="7" t="n">
-        <v>13110</v>
+        <v>37442</v>
       </c>
       <c r="D80" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E80" s="7" t="n">
-        <v>0</v>
+        <v>3581</v>
       </c>
       <c r="F80" s="7" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G80" s="7" t="n">
-        <v>0</v>
+        <v>25046</v>
       </c>
       <c r="H80" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I80" s="7" t="n">
-        <v>0</v>
+        <v>53654</v>
       </c>
       <c r="J80" s="7" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="K80" s="7" t="n">
-        <v>0</v>
+        <v>35931</v>
       </c>
       <c r="L80" s="7" t="n">
         <v>2</v>
       </c>
       <c r="M80" s="7" t="n">
-        <v>11848</v>
+        <v>23560</v>
       </c>
       <c r="N80" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O80" s="7" t="n">
-        <v>0</v>
+        <v>3749</v>
       </c>
       <c r="P80" s="7" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="Q80" s="7" t="n">
-        <v>12922</v>
+        <v>3644</v>
       </c>
       <c r="R80" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S80" s="7" t="n">
-        <v>0</v>
+        <v>623065</v>
       </c>
       <c r="T80" s="5" t="n">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="U80" s="5" t="n">
-        <v>37880</v>
+        <v>809672</v>
       </c>
     </row>
     <row r="81" ht="18" customHeight="1">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>platelet_ct</t>
+          <t>pmv</t>
         </is>
       </c>
       <c r="B81" s="7" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C81" s="7" t="n">
-        <v>37442</v>
+        <v>5707</v>
       </c>
       <c r="D81" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E81" s="7" t="n">
-        <v>3581</v>
+        <v>0</v>
       </c>
       <c r="F81" s="7" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G81" s="7" t="n">
-        <v>25046</v>
+        <v>0</v>
       </c>
       <c r="H81" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I81" s="7" t="n">
-        <v>53654</v>
+        <v>0</v>
       </c>
       <c r="J81" s="7" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="K81" s="7" t="n">
-        <v>35931</v>
+        <v>32540</v>
       </c>
       <c r="L81" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M81" s="7" t="n">
-        <v>23560</v>
+        <v>0</v>
       </c>
       <c r="N81" s="7" t="n">
         <v>1</v>
       </c>
       <c r="O81" s="7" t="n">
-        <v>3749</v>
+        <v>3376</v>
       </c>
       <c r="P81" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q81" s="7" t="n">
-        <v>3644</v>
+        <v>0</v>
       </c>
       <c r="R81" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S81" s="7" t="n">
-        <v>623065</v>
+        <v>0</v>
       </c>
       <c r="T81" s="5" t="n">
-        <v>33</v>
+        <v>8</v>
       </c>
       <c r="U81" s="5" t="n">
-        <v>809672</v>
+        <v>41623</v>
       </c>
     </row>
     <row r="82" ht="18" customHeight="1">
       <c r="A82" s="6" t="inlineStr">
         <is>
-          <t>pmv</t>
+          <t>potassium</t>
         </is>
       </c>
       <c r="B82" s="7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C82" s="7" t="n">
-        <v>5707</v>
+        <v>37384</v>
       </c>
       <c r="D82" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E82" s="7" t="n">
-        <v>0</v>
+        <v>6310</v>
       </c>
       <c r="F82" s="7" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G82" s="7" t="n">
-        <v>0</v>
+        <v>25155</v>
       </c>
       <c r="H82" s="7" t="n">
         <v>0</v>
@@ -6025,10 +6025,10 @@
         <v>0</v>
       </c>
       <c r="J82" s="7" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K82" s="7" t="n">
-        <v>32540</v>
+        <v>0</v>
       </c>
       <c r="L82" s="7" t="n">
         <v>0</v>
@@ -6040,13 +6040,13 @@
         <v>1</v>
       </c>
       <c r="O82" s="7" t="n">
-        <v>3376</v>
+        <v>3839</v>
       </c>
       <c r="P82" s="7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Q82" s="7" t="n">
-        <v>0</v>
+        <v>18964</v>
       </c>
       <c r="R82" s="7" t="n">
         <v>0</v>
@@ -6055,35 +6055,35 @@
         <v>0</v>
       </c>
       <c r="T82" s="5" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="U82" s="5" t="n">
-        <v>41623</v>
+        <v>91652</v>
       </c>
     </row>
     <row r="83" ht="18" customHeight="1">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>potassium</t>
+          <t>pr_ekg</t>
         </is>
       </c>
       <c r="B83" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C83" s="7" t="n">
-        <v>37384</v>
+        <v>59015</v>
       </c>
       <c r="D83" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E83" s="7" t="n">
-        <v>6310</v>
+        <v>0</v>
       </c>
       <c r="F83" s="7" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G83" s="7" t="n">
-        <v>25155</v>
+        <v>0</v>
       </c>
       <c r="H83" s="7" t="n">
         <v>0</v>
@@ -6098,47 +6098,47 @@
         <v>0</v>
       </c>
       <c r="L83" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M83" s="7" t="n">
-        <v>0</v>
+        <v>23526</v>
       </c>
       <c r="N83" s="7" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="O83" s="7" t="n">
-        <v>3839</v>
+        <v>78673</v>
       </c>
       <c r="P83" s="7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="Q83" s="7" t="n">
-        <v>18964</v>
+        <v>22435</v>
       </c>
       <c r="R83" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S83" s="7" t="n">
-        <v>0</v>
+        <v>500439</v>
       </c>
       <c r="T83" s="5" t="n">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="U83" s="5" t="n">
-        <v>91652</v>
+        <v>684088</v>
       </c>
     </row>
     <row r="84" ht="18" customHeight="1">
       <c r="A84" s="6" t="inlineStr">
         <is>
-          <t>pr_ekg</t>
+          <t>pr_qrs_qt</t>
         </is>
       </c>
       <c r="B84" s="7" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C84" s="7" t="n">
-        <v>59015</v>
+        <v>0</v>
       </c>
       <c r="D84" s="7" t="n">
         <v>0</v>
@@ -6159,46 +6159,46 @@
         <v>0</v>
       </c>
       <c r="J84" s="7" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="K84" s="7" t="n">
-        <v>0</v>
+        <v>66296</v>
       </c>
       <c r="L84" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M84" s="7" t="n">
-        <v>23526</v>
+        <v>0</v>
       </c>
       <c r="N84" s="7" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="O84" s="7" t="n">
-        <v>78673</v>
+        <v>0</v>
       </c>
       <c r="P84" s="7" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="Q84" s="7" t="n">
-        <v>22435</v>
+        <v>0</v>
       </c>
       <c r="R84" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S84" s="7" t="n">
-        <v>500439</v>
+        <v>0</v>
       </c>
       <c r="T84" s="5" t="n">
-        <v>42</v>
+        <v>7</v>
       </c>
       <c r="U84" s="5" t="n">
-        <v>684088</v>
+        <v>66296</v>
       </c>
     </row>
     <row r="85" ht="18" customHeight="1">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>pr_qrs_qt</t>
+          <t>pselectin</t>
         </is>
       </c>
       <c r="B85" s="7" t="n">
@@ -6208,10 +6208,10 @@
         <v>0</v>
       </c>
       <c r="D85" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E85" s="7" t="n">
-        <v>0</v>
+        <v>326</v>
       </c>
       <c r="F85" s="7" t="n">
         <v>0</v>
@@ -6226,10 +6226,10 @@
         <v>0</v>
       </c>
       <c r="J85" s="7" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="K85" s="7" t="n">
-        <v>66296</v>
+        <v>0</v>
       </c>
       <c r="L85" s="7" t="n">
         <v>0</v>
@@ -6238,10 +6238,10 @@
         <v>0</v>
       </c>
       <c r="N85" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O85" s="7" t="n">
-        <v>0</v>
+        <v>8299</v>
       </c>
       <c r="P85" s="7" t="n">
         <v>0</v>
@@ -6256,35 +6256,35 @@
         <v>0</v>
       </c>
       <c r="T85" s="5" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="U85" s="5" t="n">
-        <v>66296</v>
+        <v>8625</v>
       </c>
     </row>
     <row r="86" ht="18" customHeight="1">
       <c r="A86" s="6" t="inlineStr">
         <is>
-          <t>pselectin</t>
+          <t>qrs_ekg</t>
         </is>
       </c>
       <c r="B86" s="7" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="C86" s="7" t="n">
-        <v>0</v>
+        <v>274284</v>
       </c>
       <c r="D86" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E86" s="7" t="n">
-        <v>326</v>
+        <v>0</v>
       </c>
       <c r="F86" s="7" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G86" s="7" t="n">
-        <v>0</v>
+        <v>43430</v>
       </c>
       <c r="H86" s="7" t="n">
         <v>0</v>
@@ -6293,53 +6293,53 @@
         <v>0</v>
       </c>
       <c r="J86" s="7" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="K86" s="7" t="n">
-        <v>0</v>
+        <v>202581</v>
       </c>
       <c r="L86" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M86" s="7" t="n">
-        <v>0</v>
+        <v>23558</v>
       </c>
       <c r="N86" s="7" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="O86" s="7" t="n">
-        <v>8299</v>
+        <v>65524</v>
       </c>
       <c r="P86" s="7" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="Q86" s="7" t="n">
-        <v>0</v>
+        <v>22514</v>
       </c>
       <c r="R86" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S86" s="7" t="n">
-        <v>0</v>
+        <v>500439</v>
       </c>
       <c r="T86" s="5" t="n">
-        <v>5</v>
+        <v>139</v>
       </c>
       <c r="U86" s="5" t="n">
-        <v>8625</v>
+        <v>1132330</v>
       </c>
     </row>
     <row r="87" ht="18" customHeight="1">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>qrs_ekg</t>
+          <t>qt_ekg</t>
         </is>
       </c>
       <c r="B87" s="7" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="C87" s="7" t="n">
-        <v>274284</v>
+        <v>61199</v>
       </c>
       <c r="D87" s="7" t="n">
         <v>0</v>
@@ -6348,10 +6348,10 @@
         <v>0</v>
       </c>
       <c r="F87" s="7" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="G87" s="7" t="n">
-        <v>43430</v>
+        <v>0</v>
       </c>
       <c r="H87" s="7" t="n">
         <v>0</v>
@@ -6360,22 +6360,22 @@
         <v>0</v>
       </c>
       <c r="J87" s="7" t="n">
-        <v>75</v>
+        <v>20</v>
       </c>
       <c r="K87" s="7" t="n">
-        <v>202581</v>
+        <v>90128</v>
       </c>
       <c r="L87" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M87" s="7" t="n">
-        <v>23558</v>
+        <v>35283</v>
       </c>
       <c r="N87" s="7" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="O87" s="7" t="n">
-        <v>65524</v>
+        <v>46378</v>
       </c>
       <c r="P87" s="7" t="n">
         <v>8</v>
@@ -6390,29 +6390,29 @@
         <v>500439</v>
       </c>
       <c r="T87" s="5" t="n">
-        <v>139</v>
+        <v>54</v>
       </c>
       <c r="U87" s="5" t="n">
-        <v>1132330</v>
+        <v>755941</v>
       </c>
     </row>
     <row r="88" ht="18" customHeight="1">
       <c r="A88" s="6" t="inlineStr">
         <is>
-          <t>qt_ekg</t>
+          <t>rdbld_ct</t>
         </is>
       </c>
       <c r="B88" s="7" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C88" s="7" t="n">
-        <v>61199</v>
+        <v>14728</v>
       </c>
       <c r="D88" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E88" s="7" t="n">
-        <v>0</v>
+        <v>3583</v>
       </c>
       <c r="F88" s="7" t="n">
         <v>0</v>
@@ -6421,65 +6421,65 @@
         <v>0</v>
       </c>
       <c r="H88" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I88" s="7" t="n">
-        <v>0</v>
+        <v>53674</v>
       </c>
       <c r="J88" s="7" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="K88" s="7" t="n">
-        <v>90128</v>
+        <v>59154</v>
       </c>
       <c r="L88" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M88" s="7" t="n">
-        <v>35283</v>
+        <v>23567</v>
       </c>
       <c r="N88" s="7" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="O88" s="7" t="n">
-        <v>46378</v>
+        <v>3377</v>
       </c>
       <c r="P88" s="7" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="Q88" s="7" t="n">
-        <v>22514</v>
+        <v>3656</v>
       </c>
       <c r="R88" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S88" s="7" t="n">
-        <v>500439</v>
+        <v>0</v>
       </c>
       <c r="T88" s="5" t="n">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="U88" s="5" t="n">
-        <v>755941</v>
+        <v>161739</v>
       </c>
     </row>
     <row r="89" ht="18" customHeight="1">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>rdbld_ct</t>
+          <t>rdw</t>
         </is>
       </c>
       <c r="B89" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C89" s="7" t="n">
-        <v>14728</v>
+        <v>12016</v>
       </c>
       <c r="D89" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E89" s="7" t="n">
-        <v>3583</v>
+        <v>0</v>
       </c>
       <c r="F89" s="7" t="n">
         <v>0</v>
@@ -6488,71 +6488,71 @@
         <v>0</v>
       </c>
       <c r="H89" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I89" s="7" t="n">
-        <v>53674</v>
+        <v>0</v>
       </c>
       <c r="J89" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="K89" s="7" t="n">
+        <v>32543</v>
+      </c>
+      <c r="L89" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="M89" s="7" t="n">
+        <v>23566</v>
+      </c>
+      <c r="N89" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O89" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P89" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q89" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R89" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S89" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T89" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="K89" s="7" t="n">
-        <v>59154</v>
-      </c>
-      <c r="L89" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="M89" s="7" t="n">
-        <v>23567</v>
-      </c>
-      <c r="N89" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="O89" s="7" t="n">
-        <v>3377</v>
-      </c>
-      <c r="P89" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q89" s="7" t="n">
-        <v>3656</v>
-      </c>
-      <c r="R89" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="S89" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="T89" s="5" t="n">
-        <v>23</v>
-      </c>
       <c r="U89" s="5" t="n">
-        <v>161739</v>
+        <v>68125</v>
       </c>
     </row>
     <row r="90" ht="18" customHeight="1">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>rdw</t>
+          <t>sleep_duration_daily</t>
         </is>
       </c>
       <c r="B90" s="7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C90" s="7" t="n">
-        <v>12016</v>
+        <v>5925</v>
       </c>
       <c r="D90" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E90" s="7" t="n">
-        <v>0</v>
+        <v>3529</v>
       </c>
       <c r="F90" s="7" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G90" s="7" t="n">
-        <v>0</v>
+        <v>13853</v>
       </c>
       <c r="H90" s="7" t="n">
         <v>0</v>
@@ -6561,132 +6561,132 @@
         <v>0</v>
       </c>
       <c r="J90" s="7" t="n">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="K90" s="7" t="n">
-        <v>32543</v>
+        <v>129670</v>
       </c>
       <c r="L90" s="7" t="n">
         <v>2</v>
       </c>
       <c r="M90" s="7" t="n">
-        <v>23566</v>
+        <v>23080</v>
       </c>
       <c r="N90" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O90" s="7" t="n">
-        <v>0</v>
+        <v>6955</v>
       </c>
       <c r="P90" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q90" s="7" t="n">
-        <v>0</v>
+        <v>10941</v>
       </c>
       <c r="R90" s="7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S90" s="7" t="n">
-        <v>0</v>
+        <v>626832</v>
       </c>
       <c r="T90" s="5" t="n">
-        <v>11</v>
+        <v>55</v>
       </c>
       <c r="U90" s="5" t="n">
-        <v>68125</v>
+        <v>820785</v>
       </c>
     </row>
     <row r="91" ht="18" customHeight="1">
       <c r="A91" s="6" t="inlineStr">
         <is>
-          <t>sleep_duration_daily</t>
+          <t>sodium_blood</t>
         </is>
       </c>
       <c r="B91" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C91" s="7" t="n">
+        <v>52984</v>
+      </c>
+      <c r="D91" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E91" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F91" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G91" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H91" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I91" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J91" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="K91" s="7" t="n">
+        <v>17171</v>
+      </c>
+      <c r="L91" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M91" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N91" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="C91" s="7" t="n">
-        <v>5925</v>
-      </c>
-      <c r="D91" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E91" s="7" t="n">
-        <v>3529</v>
-      </c>
-      <c r="F91" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G91" s="7" t="n">
-        <v>13853</v>
-      </c>
-      <c r="H91" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I91" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J91" s="7" t="n">
-        <v>31</v>
-      </c>
-      <c r="K91" s="7" t="n">
-        <v>129670</v>
-      </c>
-      <c r="L91" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="M91" s="7" t="n">
-        <v>23080</v>
-      </c>
-      <c r="N91" s="7" t="n">
-        <v>2</v>
-      </c>
       <c r="O91" s="7" t="n">
-        <v>6955</v>
+        <v>3839</v>
       </c>
       <c r="P91" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q91" s="7" t="n">
-        <v>10941</v>
+        <v>6129</v>
       </c>
       <c r="R91" s="7" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="S91" s="7" t="n">
-        <v>626832</v>
+        <v>5721</v>
       </c>
       <c r="T91" s="5" t="n">
-        <v>55</v>
+        <v>11</v>
       </c>
       <c r="U91" s="5" t="n">
-        <v>820785</v>
+        <v>85844</v>
       </c>
     </row>
     <row r="92" ht="18" customHeight="1">
       <c r="A92" s="6" t="inlineStr">
         <is>
-          <t>sodium_blood</t>
+          <t>sodium_intak</t>
         </is>
       </c>
       <c r="B92" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C92" s="7" t="n">
+        <v>28614</v>
+      </c>
+      <c r="D92" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="C92" s="7" t="n">
-        <v>52984</v>
-      </c>
-      <c r="D92" s="7" t="n">
-        <v>0</v>
-      </c>
       <c r="E92" s="7" t="n">
-        <v>0</v>
+        <v>16962</v>
       </c>
       <c r="F92" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G92" s="7" t="n">
-        <v>0</v>
+        <v>12180</v>
       </c>
       <c r="H92" s="7" t="n">
         <v>0</v>
@@ -6695,10 +6695,10 @@
         <v>0</v>
       </c>
       <c r="J92" s="7" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="K92" s="7" t="n">
-        <v>17171</v>
+        <v>82860</v>
       </c>
       <c r="L92" s="7" t="n">
         <v>0</v>
@@ -6707,71 +6707,71 @@
         <v>0</v>
       </c>
       <c r="N92" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O92" s="7" t="n">
-        <v>3839</v>
+        <v>0</v>
       </c>
       <c r="P92" s="7" t="n">
         <v>1</v>
       </c>
       <c r="Q92" s="7" t="n">
-        <v>6129</v>
+        <v>4252</v>
       </c>
       <c r="R92" s="7" t="n">
         <v>1</v>
       </c>
       <c r="S92" s="7" t="n">
-        <v>5721</v>
+        <v>338044</v>
       </c>
       <c r="T92" s="5" t="n">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="U92" s="5" t="n">
-        <v>85844</v>
+        <v>482912</v>
       </c>
     </row>
     <row r="93" ht="18" customHeight="1">
       <c r="A93" s="6" t="inlineStr">
         <is>
-          <t>sodium_intak</t>
+          <t>spo2</t>
         </is>
       </c>
       <c r="B93" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C93" s="7" t="n">
-        <v>28614</v>
+        <v>0</v>
       </c>
       <c r="D93" s="7" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E93" s="7" t="n">
-        <v>16962</v>
+        <v>0</v>
       </c>
       <c r="F93" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G93" s="7" t="n">
-        <v>12180</v>
+        <v>10480</v>
       </c>
       <c r="H93" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I93" s="7" t="n">
-        <v>0</v>
+        <v>64224</v>
       </c>
       <c r="J93" s="7" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="K93" s="7" t="n">
-        <v>82860</v>
+        <v>715</v>
       </c>
       <c r="L93" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M93" s="7" t="n">
-        <v>0</v>
+        <v>22347</v>
       </c>
       <c r="N93" s="7" t="n">
         <v>0</v>
@@ -6780,28 +6780,28 @@
         <v>0</v>
       </c>
       <c r="P93" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q93" s="7" t="n">
-        <v>4252</v>
+        <v>0</v>
       </c>
       <c r="R93" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S93" s="7" t="n">
-        <v>338044</v>
+        <v>0</v>
       </c>
       <c r="T93" s="5" t="n">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="U93" s="5" t="n">
-        <v>482912</v>
+        <v>97766</v>
       </c>
     </row>
     <row r="94" ht="18" customHeight="1">
       <c r="A94" s="6" t="inlineStr">
         <is>
-          <t>spo2</t>
+          <t>tnfa</t>
         </is>
       </c>
       <c r="B94" s="7" t="n">
@@ -6817,28 +6817,28 @@
         <v>0</v>
       </c>
       <c r="F94" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G94" s="7" t="n">
-        <v>10480</v>
+        <v>0</v>
       </c>
       <c r="H94" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I94" s="7" t="n">
-        <v>64224</v>
+        <v>0</v>
       </c>
       <c r="J94" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K94" s="7" t="n">
-        <v>715</v>
+        <v>0</v>
       </c>
       <c r="L94" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M94" s="7" t="n">
-        <v>22347</v>
+        <v>0</v>
       </c>
       <c r="N94" s="7" t="n">
         <v>0</v>
@@ -6847,10 +6847,10 @@
         <v>0</v>
       </c>
       <c r="P94" s="7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Q94" s="7" t="n">
-        <v>0</v>
+        <v>6524</v>
       </c>
       <c r="R94" s="7" t="n">
         <v>0</v>
@@ -6859,16 +6859,16 @@
         <v>0</v>
       </c>
       <c r="T94" s="5" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="U94" s="5" t="n">
-        <v>97766</v>
+        <v>6524</v>
       </c>
     </row>
     <row r="95" ht="18" customHeight="1">
       <c r="A95" s="6" t="inlineStr">
         <is>
-          <t>tnfa</t>
+          <t>tnfa_r1</t>
         </is>
       </c>
       <c r="B95" s="7" t="n">
@@ -6914,10 +6914,10 @@
         <v>0</v>
       </c>
       <c r="P95" s="7" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="Q95" s="7" t="n">
-        <v>6524</v>
+        <v>9242</v>
       </c>
       <c r="R95" s="7" t="n">
         <v>0</v>
@@ -6926,35 +6926,35 @@
         <v>0</v>
       </c>
       <c r="T95" s="5" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="U95" s="5" t="n">
-        <v>6524</v>
+        <v>9242</v>
       </c>
     </row>
     <row r="96" ht="18" customHeight="1">
       <c r="A96" s="6" t="inlineStr">
         <is>
-          <t>tnfa_r1</t>
+          <t>tot_chol_bld</t>
         </is>
       </c>
       <c r="B96" s="7" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="C96" s="7" t="n">
-        <v>0</v>
+        <v>245458</v>
       </c>
       <c r="D96" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E96" s="7" t="n">
-        <v>0</v>
+        <v>6897</v>
       </c>
       <c r="F96" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G96" s="7" t="n">
-        <v>0</v>
+        <v>11010</v>
       </c>
       <c r="H96" s="7" t="n">
         <v>0</v>
@@ -6963,65 +6963,65 @@
         <v>0</v>
       </c>
       <c r="J96" s="7" t="n">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="K96" s="7" t="n">
-        <v>0</v>
+        <v>218271</v>
       </c>
       <c r="L96" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M96" s="7" t="n">
-        <v>0</v>
+        <v>23653</v>
       </c>
       <c r="N96" s="7" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="O96" s="7" t="n">
-        <v>0</v>
+        <v>31460</v>
       </c>
       <c r="P96" s="7" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="Q96" s="7" t="n">
-        <v>9242</v>
+        <v>68149</v>
       </c>
       <c r="R96" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S96" s="7" t="n">
-        <v>0</v>
+        <v>46610</v>
       </c>
       <c r="T96" s="5" t="n">
-        <v>2</v>
+        <v>131</v>
       </c>
       <c r="U96" s="5" t="n">
-        <v>9242</v>
+        <v>651508</v>
       </c>
     </row>
     <row r="97" ht="18" customHeight="1">
       <c r="A97" s="6" t="inlineStr">
         <is>
-          <t>tot_chol_bld</t>
+          <t>triglyc_bld</t>
         </is>
       </c>
       <c r="B97" s="7" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="C97" s="7" t="n">
-        <v>245458</v>
+        <v>167017</v>
       </c>
       <c r="D97" s="7" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E97" s="7" t="n">
-        <v>6897</v>
+        <v>16569</v>
       </c>
       <c r="F97" s="7" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G97" s="7" t="n">
-        <v>11010</v>
+        <v>29264</v>
       </c>
       <c r="H97" s="7" t="n">
         <v>0</v>
@@ -7030,10 +7030,10 @@
         <v>0</v>
       </c>
       <c r="J97" s="7" t="n">
-        <v>64</v>
+        <v>50</v>
       </c>
       <c r="K97" s="7" t="n">
-        <v>218271</v>
+        <v>168009</v>
       </c>
       <c r="L97" s="7" t="n">
         <v>2</v>
@@ -7042,16 +7042,16 @@
         <v>23653</v>
       </c>
       <c r="N97" s="7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="O97" s="7" t="n">
-        <v>31460</v>
+        <v>32777</v>
       </c>
       <c r="P97" s="7" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="Q97" s="7" t="n">
-        <v>68149</v>
+        <v>67803</v>
       </c>
       <c r="R97" s="7" t="n">
         <v>3</v>
@@ -7060,102 +7060,102 @@
         <v>46610</v>
       </c>
       <c r="T97" s="5" t="n">
-        <v>131</v>
+        <v>117</v>
       </c>
       <c r="U97" s="5" t="n">
-        <v>651508</v>
+        <v>551702</v>
       </c>
     </row>
     <row r="98" ht="18" customHeight="1">
       <c r="A98" s="6" t="inlineStr">
         <is>
-          <t>triglyc_bld</t>
+          <t>troponin</t>
         </is>
       </c>
       <c r="B98" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="C98" s="7" t="n">
+        <v>59241</v>
+      </c>
+      <c r="D98" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E98" s="7" t="n">
+        <v>77</v>
+      </c>
+      <c r="F98" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G98" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H98" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I98" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J98" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="K98" s="7" t="n">
+        <v>14391</v>
+      </c>
+      <c r="L98" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M98" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N98" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O98" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P98" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q98" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R98" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="S98" s="7" t="n">
+        <v>4604</v>
+      </c>
+      <c r="T98" s="5" t="n">
         <v>18</v>
       </c>
-      <c r="C98" s="7" t="n">
-        <v>167017</v>
-      </c>
-      <c r="D98" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="E98" s="7" t="n">
-        <v>16569</v>
-      </c>
-      <c r="F98" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="G98" s="7" t="n">
-        <v>29264</v>
-      </c>
-      <c r="H98" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I98" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J98" s="7" t="n">
-        <v>50</v>
-      </c>
-      <c r="K98" s="7" t="n">
-        <v>168009</v>
-      </c>
-      <c r="L98" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="M98" s="7" t="n">
-        <v>23653</v>
-      </c>
-      <c r="N98" s="7" t="n">
-        <v>13</v>
-      </c>
-      <c r="O98" s="7" t="n">
-        <v>32777</v>
-      </c>
-      <c r="P98" s="7" t="n">
-        <v>19</v>
-      </c>
-      <c r="Q98" s="7" t="n">
-        <v>67803</v>
-      </c>
-      <c r="R98" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="S98" s="7" t="n">
-        <v>46610</v>
-      </c>
-      <c r="T98" s="5" t="n">
-        <v>117</v>
-      </c>
       <c r="U98" s="5" t="n">
-        <v>551702</v>
+        <v>78313</v>
       </c>
     </row>
     <row r="99" ht="18" customHeight="1">
       <c r="A99" s="6" t="inlineStr">
         <is>
-          <t>troponin</t>
+          <t>vege_serving</t>
         </is>
       </c>
       <c r="B99" s="7" t="n">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="C99" s="7" t="n">
-        <v>59241</v>
+        <v>322380</v>
       </c>
       <c r="D99" s="7" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="E99" s="7" t="n">
-        <v>77</v>
+        <v>74514</v>
       </c>
       <c r="F99" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G99" s="7" t="n">
-        <v>0</v>
+        <v>771</v>
       </c>
       <c r="H99" s="7" t="n">
         <v>0</v>
@@ -7164,10 +7164,10 @@
         <v>0</v>
       </c>
       <c r="J99" s="7" t="n">
-        <v>4</v>
+        <v>232</v>
       </c>
       <c r="K99" s="7" t="n">
-        <v>14391</v>
+        <v>638568</v>
       </c>
       <c r="L99" s="7" t="n">
         <v>0</v>
@@ -7176,429 +7176,362 @@
         <v>0</v>
       </c>
       <c r="N99" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O99" s="7" t="n">
-        <v>0</v>
+        <v>7594</v>
       </c>
       <c r="P99" s="7" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="Q99" s="7" t="n">
-        <v>0</v>
+        <v>29869</v>
       </c>
       <c r="R99" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S99" s="7" t="n">
-        <v>4604</v>
+        <v>680137</v>
       </c>
       <c r="T99" s="5" t="n">
-        <v>18</v>
+        <v>300</v>
       </c>
       <c r="U99" s="5" t="n">
-        <v>78313</v>
+        <v>1753833</v>
       </c>
     </row>
     <row r="100" ht="18" customHeight="1">
       <c r="A100" s="6" t="inlineStr">
         <is>
-          <t>vege_serving</t>
+          <t>waist_circ</t>
         </is>
       </c>
       <c r="B100" s="7" t="n">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="C100" s="7" t="n">
-        <v>322380</v>
+        <v>54019</v>
       </c>
       <c r="D100" s="7" t="n">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="E100" s="7" t="n">
-        <v>74514</v>
+        <v>30185</v>
       </c>
       <c r="F100" s="7" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="G100" s="7" t="n">
-        <v>771</v>
+        <v>43939</v>
       </c>
       <c r="H100" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I100" s="7" t="n">
-        <v>0</v>
+        <v>53850</v>
       </c>
       <c r="J100" s="7" t="n">
-        <v>232</v>
+        <v>55</v>
       </c>
       <c r="K100" s="7" t="n">
-        <v>638568</v>
+        <v>175209</v>
       </c>
       <c r="L100" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M100" s="7" t="n">
-        <v>0</v>
+        <v>23633</v>
       </c>
       <c r="N100" s="7" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="O100" s="7" t="n">
-        <v>7594</v>
+        <v>25409</v>
       </c>
       <c r="P100" s="7" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="Q100" s="7" t="n">
-        <v>29869</v>
+        <v>56543</v>
       </c>
       <c r="R100" s="7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="S100" s="7" t="n">
-        <v>680137</v>
+        <v>1619039</v>
       </c>
       <c r="T100" s="5" t="n">
-        <v>300</v>
+        <v>112</v>
       </c>
       <c r="U100" s="5" t="n">
-        <v>1753833</v>
+        <v>2081826</v>
       </c>
     </row>
     <row r="101" ht="18" customHeight="1">
       <c r="A101" s="6" t="inlineStr">
         <is>
-          <t>waist_circ</t>
+          <t>waist_hip</t>
         </is>
       </c>
       <c r="B101" s="7" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C101" s="7" t="n">
-        <v>54019</v>
+        <v>106654</v>
       </c>
       <c r="D101" s="7" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="E101" s="7" t="n">
-        <v>30185</v>
+        <v>388</v>
       </c>
       <c r="F101" s="7" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="G101" s="7" t="n">
-        <v>43939</v>
+        <v>0</v>
       </c>
       <c r="H101" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I101" s="7" t="n">
-        <v>53850</v>
+        <v>0</v>
       </c>
       <c r="J101" s="7" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="K101" s="7" t="n">
-        <v>175209</v>
+        <v>0</v>
       </c>
       <c r="L101" s="7" t="n">
         <v>2</v>
       </c>
       <c r="M101" s="7" t="n">
-        <v>23633</v>
+        <v>23626</v>
       </c>
       <c r="N101" s="7" t="n">
         <v>8</v>
       </c>
       <c r="O101" s="7" t="n">
-        <v>25409</v>
+        <v>23478</v>
       </c>
       <c r="P101" s="7" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="Q101" s="7" t="n">
-        <v>56543</v>
+        <v>89497</v>
       </c>
       <c r="R101" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S101" s="7" t="n">
-        <v>1619039</v>
+        <v>1610605</v>
       </c>
       <c r="T101" s="5" t="n">
-        <v>112</v>
+        <v>51</v>
       </c>
       <c r="U101" s="5" t="n">
-        <v>2081826</v>
+        <v>1854248</v>
       </c>
     </row>
     <row r="102" ht="18" customHeight="1">
       <c r="A102" s="6" t="inlineStr">
         <is>
-          <t>waist_hip</t>
+          <t>whtbld_ct</t>
         </is>
       </c>
       <c r="B102" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C102" s="7" t="n">
+        <v>43076</v>
+      </c>
+      <c r="D102" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E102" s="7" t="n">
+        <v>3583</v>
+      </c>
+      <c r="F102" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G102" s="7" t="n">
+        <v>10978</v>
+      </c>
+      <c r="H102" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="I102" s="7" t="n">
+        <v>53674</v>
+      </c>
+      <c r="J102" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="C102" s="7" t="n">
-        <v>106654</v>
-      </c>
-      <c r="D102" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E102" s="7" t="n">
-        <v>388</v>
-      </c>
-      <c r="F102" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G102" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H102" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I102" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J102" s="7" t="n">
-        <v>0</v>
-      </c>
       <c r="K102" s="7" t="n">
-        <v>0</v>
+        <v>60160</v>
       </c>
       <c r="L102" s="7" t="n">
         <v>2</v>
       </c>
       <c r="M102" s="7" t="n">
-        <v>23626</v>
+        <v>22911</v>
       </c>
       <c r="N102" s="7" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="O102" s="7" t="n">
-        <v>23478</v>
+        <v>3377</v>
       </c>
       <c r="P102" s="7" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="Q102" s="7" t="n">
-        <v>89497</v>
+        <v>3656</v>
       </c>
       <c r="R102" s="7" t="n">
         <v>3</v>
       </c>
       <c r="S102" s="7" t="n">
-        <v>1610605</v>
+        <v>623680</v>
       </c>
       <c r="T102" s="5" t="n">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="U102" s="5" t="n">
-        <v>1854248</v>
+        <v>825095</v>
       </c>
     </row>
     <row r="103" ht="18" customHeight="1">
       <c r="A103" s="6" t="inlineStr">
         <is>
-          <t>whtbld_ct</t>
+          <t>willeb_fac</t>
         </is>
       </c>
       <c r="B103" s="7" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C103" s="7" t="n">
-        <v>43076</v>
+        <v>14801</v>
       </c>
       <c r="D103" s="7" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E103" s="7" t="n">
-        <v>3583</v>
+        <v>6928</v>
       </c>
       <c r="F103" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G103" s="7" t="n">
-        <v>10978</v>
+        <v>0</v>
       </c>
       <c r="H103" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I103" s="7" t="n">
-        <v>53674</v>
+        <v>0</v>
       </c>
       <c r="J103" s="7" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="K103" s="7" t="n">
-        <v>60160</v>
+        <v>12072</v>
       </c>
       <c r="L103" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M103" s="7" t="n">
-        <v>22911</v>
+        <v>0</v>
       </c>
       <c r="N103" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O103" s="7" t="n">
-        <v>3377</v>
+        <v>0</v>
       </c>
       <c r="P103" s="7" t="n">
         <v>2</v>
       </c>
       <c r="Q103" s="7" t="n">
-        <v>3656</v>
+        <v>7391</v>
       </c>
       <c r="R103" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S103" s="7" t="n">
-        <v>623680</v>
+        <v>0</v>
       </c>
       <c r="T103" s="5" t="n">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="U103" s="5" t="n">
-        <v>825095</v>
+        <v>41192</v>
       </c>
     </row>
     <row r="104" ht="18" customHeight="1">
-      <c r="A104" s="6" t="inlineStr">
-        <is>
-          <t>willeb_fac</t>
-        </is>
-      </c>
-      <c r="B104" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C104" s="7" t="n">
-        <v>14801</v>
-      </c>
-      <c r="D104" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="E104" s="7" t="n">
-        <v>6928</v>
-      </c>
-      <c r="F104" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G104" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H104" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I104" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J104" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="K104" s="7" t="n">
-        <v>12072</v>
-      </c>
-      <c r="L104" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M104" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N104" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O104" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P104" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q104" s="7" t="n">
-        <v>7391</v>
-      </c>
-      <c r="R104" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="S104" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="T104" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="U104" s="5" t="n">
-        <v>41192</v>
-      </c>
-    </row>
-    <row r="105" ht="18" customHeight="1">
-      <c r="A105" s="8" t="inlineStr">
+      <c r="A104" s="8" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B105" s="9" t="n">
+      <c r="B104" s="9" t="n">
         <v>1167</v>
       </c>
-      <c r="C105" s="9" t="n">
+      <c r="C104" s="9" t="n">
         <v>11476318</v>
       </c>
-      <c r="D105" s="9" t="n">
+      <c r="D104" s="9" t="n">
         <v>551</v>
       </c>
-      <c r="E105" s="9" t="n">
+      <c r="E104" s="9" t="n">
         <v>1001601</v>
       </c>
-      <c r="F105" s="9" t="n">
+      <c r="F104" s="9" t="n">
         <v>1341</v>
       </c>
-      <c r="G105" s="9" t="n">
+      <c r="G104" s="9" t="n">
         <v>4128699</v>
       </c>
-      <c r="H105" s="9" t="n">
+      <c r="H104" s="9" t="n">
         <v>108</v>
       </c>
-      <c r="I105" s="9" t="n">
+      <c r="I104" s="9" t="n">
         <v>2062015</v>
       </c>
-      <c r="J105" s="9" t="n">
+      <c r="J104" s="9" t="n">
         <v>3058</v>
       </c>
-      <c r="K105" s="9" t="n">
+      <c r="K104" s="9" t="n">
         <v>9163012</v>
       </c>
-      <c r="L105" s="9" t="n">
+      <c r="L104" s="9" t="n">
         <v>163</v>
       </c>
-      <c r="M105" s="9" t="n">
+      <c r="M104" s="9" t="n">
         <v>1749972</v>
       </c>
-      <c r="N105" s="9" t="n">
+      <c r="N104" s="9" t="n">
         <v>476</v>
       </c>
-      <c r="O105" s="9" t="n">
+      <c r="O104" s="9" t="n">
         <v>1639132</v>
       </c>
-      <c r="P105" s="9" t="n">
+      <c r="P104" s="9" t="n">
         <v>1183</v>
       </c>
-      <c r="Q105" s="9" t="n">
+      <c r="Q104" s="9" t="n">
         <v>3873029</v>
       </c>
-      <c r="R105" s="9" t="n">
+      <c r="R104" s="9" t="n">
         <v>353</v>
       </c>
-      <c r="S105" s="9" t="n">
+      <c r="S104" s="9" t="n">
         <v>33610590</v>
       </c>
-      <c r="T105" s="9" t="n">
+      <c r="T104" s="9" t="n">
         <v>8400</v>
       </c>
-      <c r="U105" s="9" t="n">
+      <c r="U104" s="9" t="n">
         <v>68704368</v>
       </c>
     </row>

</xml_diff>